<commit_message>
Tester guide section 13 (R3 deploy 1) and refreshed workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/MIS_TESTER_TRACKER.xlsx
+++ b/docs/qa/MIS_TESTER_TRACKER.xlsx
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2172,7 +2172,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C45" s="3" t="n"/>
+      <c r="C45" s="3" t="inlineStr"/>
       <c r="D45" s="3" t="inlineStr">
         <is>
           <t>Health screen (hold the top bar 3 s) → sync</t>
@@ -2202,7 +2202,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C46" s="3" t="n"/>
+      <c r="C46" s="3" t="inlineStr"/>
       <c r="D46" s="3" t="inlineStr">
         <is>
           <t>Sign in as operator using an **ordinary worker's** badge code</t>
@@ -2232,7 +2232,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C47" s="3" t="n"/>
+      <c r="C47" s="3" t="inlineStr"/>
       <c r="D47" s="3" t="inlineStr">
         <is>
           <t>Sign in using the **operator's** badge code</t>
@@ -2262,7 +2262,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C48" s="3" t="n"/>
+      <c r="C48" s="3" t="inlineStr"/>
       <c r="D48" s="3" t="inlineStr">
         <is>
           <t>Right after sign-in</t>
@@ -2292,7 +2292,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C49" s="3" t="n"/>
+      <c r="C49" s="3" t="inlineStr"/>
       <c r="D49" s="3" t="inlineStr">
         <is>
           <t>Pick a shift</t>
@@ -2322,7 +2322,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C50" s="3" t="n"/>
+      <c r="C50" s="3" t="inlineStr"/>
       <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Scan the badge (QR) of a worker **with** a photo</t>
@@ -2352,7 +2352,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C51" s="3" t="n"/>
+      <c r="C51" s="3" t="inlineStr"/>
       <c r="D51" s="3" t="inlineStr">
         <is>
           <t>Scan a worker **without** a photo</t>
@@ -2382,7 +2382,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C52" s="3" t="n"/>
+      <c r="C52" s="3" t="inlineStr"/>
       <c r="D52" s="3" t="inlineStr">
         <is>
           <t>Type the worker's code manually instead of scanning</t>
@@ -2412,7 +2412,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C53" s="3" t="n"/>
+      <c r="C53" s="3" t="inlineStr"/>
       <c r="D53" s="3" t="inlineStr">
         <is>
           <t>Punch several workers in, then out</t>
@@ -2442,7 +2442,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C54" s="3" t="n"/>
+      <c r="C54" s="3" t="inlineStr"/>
       <c r="D54" s="3" t="inlineStr">
         <is>
           <t>Wifi off → punch 2–3 workers → wifi on</t>
@@ -2472,7 +2472,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C55" s="3" t="n"/>
+      <c r="C55" s="3" t="inlineStr"/>
       <c r="D55" s="3" t="inlineStr">
         <is>
           <t>Wifi off → scan a worker with a photo</t>
@@ -2502,7 +2502,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C56" s="3" t="n"/>
+      <c r="C56" s="3" t="inlineStr"/>
       <c r="D56" s="3" t="inlineStr">
         <is>
           <t>Health screen → **End shift**</t>
@@ -2532,7 +2532,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C57" s="3" t="n"/>
+      <c r="C57" s="3" t="inlineStr"/>
       <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Close and reopen the app while signed in</t>
@@ -2562,7 +2562,7 @@
           <t>§7. Android kiosk (needs the NEW APK, October 2026 build)</t>
         </is>
       </c>
-      <c r="C58" s="3" t="n"/>
+      <c r="C58" s="3" t="inlineStr"/>
       <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Web: Settings → Gate tablets → revoke this tablet</t>
@@ -4246,6 +4246,822 @@
       </c>
       <c r="G107" s="3" t="n"/>
       <c r="H107" s="3" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>STORE_GUY</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>GRN receiving 2% over the PO qty, then 3% over</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>2% allowed; 3% refused with the max shown</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="n"/>
+      <c r="H108" s="3" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>STORE_GUY</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>Receive the last of a PO</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>PO shows COMPLETE and leaves the GRN picker</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="n"/>
+      <c r="H109" s="3" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>STORE_GUY</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Issue more than stock; double-tap Confirm on the cart</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>Refused; books once</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="n"/>
+      <c r="H110" s="3" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>13.4</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>STORE_GUY</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>Inventory adjust without a reason</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>Reason required (3+ characters)</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="n"/>
+      <c r="H111" s="3" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>13.5</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>STORE_GUY</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>Orders / Customers / Dashboard / Order detail</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>All open, read-only, no prices, no error page</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="n"/>
+      <c r="H112" s="3" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>13.6</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>Over-receipt override</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>Needs a reason</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="n"/>
+      <c r="H113" s="3" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>13.7</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>Create a PO line with a rate</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>Rate ignored (unpriced); PO needs Owner approval</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="n"/>
+      <c r="H114" s="3" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>Approve that PO</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>Refused until every line is priced; Owner can set rates while PENDING</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="n"/>
+      <c r="H115" s="3" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>13.9</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>Change an employee wage code / pay type; deactivate the Owner row; assign Admin role</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>All refused</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="n"/>
+      <c r="H116" s="3" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>13.10</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>Business rules (PO approval threshold)</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>Not editable by Admin</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="n"/>
+      <c r="H117" s="3" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>13.11</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>Import a sheet with Name + Code only</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>Category and unit unchanged</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="n"/>
+      <c r="H118" s="3" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>13.12</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>New item</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>Next ITM- code; code editable; GSM / Size / Unit are dropdowns</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="n"/>
+      <c r="H119" s="3" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>13.13</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN / OWNER</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>Cancel an order with a machine and crew booked</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>Machine and crew freed; stock reservations released</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="n"/>
+      <c r="H120" s="3" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>13.14</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>Complete an order with no production logged</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>Refused unless Owner/Admin override with reason</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="n"/>
+      <c r="H121" s="3" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>13.15</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>Payroll for a month incl. MONTHLY staff with no attendance; department extra-pay day; half-day festival pay; closing a future month</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>Staff listed; dept day paid; half pay; future close refused</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G122" s="3" t="n"/>
+      <c r="H122" s="3" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>13.16</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Legacy issues report</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>Lists the old STORE_ISSUE rows (about 36)</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="n"/>
+      <c r="H123" s="3" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>13.17</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>CoA for an order whose failure was later fixed; for a non-completed order</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>PASS; DRAFT banner</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="n"/>
+      <c r="H124" s="3" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>13.18</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>Crew: staff tomorrow, move a worker, assign someone on leave or double-booked, copy yesterday</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>Works; overlap and leave blocked (Admin can override with reason)</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="n"/>
+      <c r="H125" s="3" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>13.19</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>Sign off a phase</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>Machine AND crew freed</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="n"/>
+      <c r="H126" s="3" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>13.20</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>Production entry: edit within 24h; log on an unbooked machine; mixed units</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>Edit works then refused; amber warning; totals per unit</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="n"/>
+      <c r="H127" s="3" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>13.21</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>Add an attendance note; add a QC check</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>Allowed</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G128" s="3" t="n"/>
+      <c r="H128" s="3" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>13.22</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>AQL sample size 0; edit a check within 24h; pass rate with N/A rows</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>Refused; allowed; N/A ignored</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="n"/>
+      <c r="H129" s="3" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>13.23</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>ATTENDANCE</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>Duplicate leave; self-approve leave; mark-absent after punches; edit outside the correction window</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>Refused; skips people who punched; refused</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="n"/>
+      <c r="H130" s="3" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>13.24</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>§13. Round 4 (R3 deploy 1) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>KIOSK (new APK)</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>Night-shift worker at 05:30; revoked tablet with queued punches; stuck entry</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>Defaults to OUT; queued punches sent before wipe; stuck row listed with Retry</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="n"/>
+      <c r="H131" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
@@ -4421,7 +5237,7 @@
           <t>Only the "Approve" button is present. There is no Reject/Return to Draft button in the UI, and no `rejectBom` server action exists in the backend. Once submitted, the BOM is locked in PENDING_APPROVAL and cannot be edited or sent back for revisions.</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -4489,7 +5305,7 @@
           <t>`gsm`, `size`, `substrate`, and `coating` are rendered as free-text input boxes (`type: 'text'`), completely disconnected from the `MisMasterOption` tables. Furthermore, `unit` uses a static hardcoded array instead of reading from the `UNIT` master options. This causes severe data inconsistency (e.g., users typing "300", "300 GSM", "300gsm", or varying size formats) and defeats the purpose of maintaining option masters.</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -4500,7 +5316,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="n"/>
       <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
     </row>
@@ -4553,7 +5369,7 @@
           <t>There is no "Delete BOM" option anywhere on the screen. The user has to manually delete every single stage and material one by one, and even then the empty BOM container permanently remains attached to the order.</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -4621,7 +5437,7 @@
           <t>The PO header card is completely read-only. There is no edit button or modal available. Only individual line items can be added/removed, but mistake in header requires cancelling the PO and making a fresh one.</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="n"/>
       <c r="K5" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -4688,7 +5504,7 @@
           <t>Only the "Cancel" button is available, which marks the draft PO as `CANCELLED`. This permanently clutters the PO listing table with junk/mistake records instead of cleaning them up.</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -4758,7 +5574,7 @@
           <t>The empty PO with 0 items and ₹0 value was successfully submitted and approved by Admin/Owner, resulting in an invalid `APPROVED` PO in the system that causes errors during GRN receipt creation.</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -4827,7 +5643,7 @@
           <t>The server action threw `500 Internal Server Error` (`POST /mis/po`), and the entire page crashed to the Next.js Error Boundary showing the "Something went wrong" screen.</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="n"/>
       <c r="K8" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -4895,7 +5711,7 @@
           <t>"BOM Ref" is rendered as an unvalidated free-text input box (`&lt;input type="text"&gt;`). The user has to manually memorize and type the reference string, which has no validation against existing BOMs and easily leads to typos, broken traceability, and orphan records.</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -4964,7 +5780,7 @@
           <t>The system allowed the PO to be created against a `DRAFT` / `PENDING_APPROVAL` BOM without any restriction or warning, creating financial risk of purchasing incorrect raw materials before technical recipe approval.</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5031,7 +5847,7 @@
           <t>There is no "Edit" option for stages or materials. Only "Remove" (delete) and "+ Add" are available. A typo in quantity or rate forces the user to completely delete the item and re-enter all details from scratch.</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5099,7 +5915,7 @@
           <t>There are no Edit or Remove buttons on the added item cards. Once an item is added, its quantity and batch number cannot be edited or deleted in UI, forcing the user to confirm with wrong quantities or leave the draft orphaned.</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5167,7 +5983,7 @@
           <t>The "PO Line Item" dropdown completely hides and removes any PO item once it is added once (`availablePoItems` filters out `addedPoItemIds`), making multi-batch / multi-reel receipt impossible in a single GRN.</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="n"/>
       <c r="K13" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5234,7 +6050,7 @@
           <t>There is no delete, cancel, or discard action on `/mis/grn/[id]` or `/mis/grn`. The draft GRN permanently remains in the system and cannot be cleaned up.</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5302,7 +6118,7 @@
           <t>Backend `confirmGRN` silently executes `if (!grnItem.poItem.itemId) continue;`, confirming the GRN as successful but silently skipping the inventory ledger insertion. Zero stock is added to warehouse balance with no warning shown to the store keeper.</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5369,7 +6185,7 @@
           <t>The system accepted negative/zero quantities and passed them to `misInventoryLedger`, deducting stock on a receipt transaction and corrupting warehouse ledger balance.</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="n"/>
       <c r="K16" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5438,7 +6254,7 @@
 2. On `/mis/production/[id]`, the unit field is an unvalidated free-text input box where users can type arbitrary strings (`kg`, `KG`, `pcs`, `sheets`), creating inconsistent data and broken aggregations.</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="n"/>
       <c r="K17" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5506,7 +6322,7 @@
           <t>There are no Action buttons (no Edit and no Delete) on the Production Log table, and backend lacks `updateProductionLog` / `deleteProductionLog` functions. Incorrect entries cannot be corrected, permanently corrupting order progress, waste rate %, and plant production metrics.</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="n"/>
       <c r="K18" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5517,7 +6333,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr"/>
+      <c r="M18" s="3" t="n"/>
       <c r="N18" s="3" t="n"/>
       <c r="O18" s="3" t="n"/>
     </row>
@@ -5569,7 +6385,7 @@
           <t>There is no Stage or Process selection in the UI. The log is created without stage association, making it impossible to track stage-wise output, bottlenecks, or stage-wise scrap rates.</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5637,7 +6453,7 @@
           <t>The dropdown renders only raw, unadorned employee names without Role, Department, or Employee Code. Non-floor roles (such as "Arjun Admin") are mixed into the list, making it confusing and error-prone for supervisors to identify and assign the correct machine operators.</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="n"/>
       <c r="K20" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5705,7 +6521,7 @@
           <t>`/mis/grn` confirmation writes exclusively to `mis_inventory_ledger` and completely fails to write to `mis_store_transactions`. As a result, `/mis/store/stock` displays 0 balance, and `/mis/store/issue` flags the item as "Out of stock" (refusing to issue it to production).</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="n"/>
       <c r="K21" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5773,7 +6589,7 @@
           <t>`recordPhysicalCount` only creates an audit log in `mis_physical_count` and never adjusts the stock balance. The system balance continues to show 500 KG, making the physical stock-taking feature purely decorative without stock reconciliation.</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="n"/>
       <c r="K22" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5841,7 +6657,7 @@
           <t>`/mis/store/transactions` allows negative balances (`isOverIssue = true`), whereas `/mis/store/issue` strictly throws an unhandled error (`Cannot issue more than the stock balance`), and `/mis/inventory` throws `Adjustment would result in negative balance`. The system has conflicting business logic across different screens.</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="n"/>
       <c r="K23" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5908,7 +6724,7 @@
           <t>The units are hardcoded to a static Prisma enum (`PIECE`, `KG`, `LITRE`, `REAM`). Users cannot create items with standard packaging units like `SHEETS` or `BOXES`, leading to unit mismatch across BOM and Store.</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="n"/>
       <c r="K24" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -5919,7 +6735,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr"/>
+      <c r="M24" s="3" t="n"/>
       <c r="N24" s="3" t="n"/>
       <c r="O24" s="3" t="n"/>
     </row>
@@ -5975,7 +6791,7 @@
           <t>There are no navigation buttons for Issue, Receive, or Physical Count anywhere on `/mis/store` or `/mis/store/dashboard`. These critical features are completely hidden/orphaned and can only be accessed by manually typing URLs in the browser address bar.</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="n"/>
       <c r="K25" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6042,7 +6858,7 @@
           <t>There are no breadcrumbs or back navigation buttons. The user is left trapped on the cart screen with no way to return to Store Stock or Overview other than clicking the global sidebar or using the browser's back button.</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="n"/>
       <c r="K26" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6077,13 +6893,13 @@
           <t>Deferred</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr"/>
-      <c r="J27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
       <c r="K27" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6094,7 +6910,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M27" s="3" t="inlineStr"/>
+      <c r="M27" s="3" t="n"/>
       <c r="N27" s="3" t="n"/>
       <c r="O27" s="3" t="n"/>
     </row>
@@ -6114,13 +6930,13 @@
           <t>Fixed - Ready to Retest</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr"/>
-      <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
       <c r="K28" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6188,7 +7004,7 @@
           <t>There is no button or dropdown anywhere in the UI to change an order's status to `COMPLETE`. The only button available is "Confirm" (from `DRAFT` to `CONFIRMED`). Once confirmed, the order is permanently stuck in `CONFIRMED` status with no way to mark it complete.</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="n"/>
       <c r="K29" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6257,7 +7073,7 @@
           <t>Backend `updateOrderStatus` accepts any arbitrary string with zero business validation. An order with zero produced items and failing QC can be transitioned directly to `COMPLETE`, bypassing all manufacturing quality gates.</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="n"/>
       <c r="K30" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6325,7 +7141,7 @@
           <t>There is no Stage dropdown in the modal form. All checks submitted through this modal are saved with `bomStageId = undefined`, rendering as empty dashes (`Stage: —`) in the QC table and making stage-wise quality tracking impossible.</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="n"/>
       <c r="K31" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6392,7 +7208,7 @@
           <t>There are no Action buttons (no Edit and no Delete) on the QC Checks table, and backend lacks `updateQcCheck` and `deleteQcCheck` functions. A mistaken check permanently taints the order's pass rate and triggers false supervisor defect notifications.</t>
         </is>
       </c>
-      <c r="J32" s="3" t="inlineStr"/>
+      <c r="J32" s="3" t="n"/>
       <c r="K32" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6403,7 +7219,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr"/>
+      <c r="M32" s="3" t="n"/>
       <c r="N32" s="3" t="n"/>
       <c r="O32" s="3" t="n"/>
     </row>
@@ -6458,7 +7274,7 @@
 2. If store issuance was recorded via Store Transactions (`createStoreOut`), it fails to populate `mis_inventory_ledger`, causing the "Material Issued" section in Traceability to show "None", breaking the audit trail.</t>
         </is>
       </c>
-      <c r="J33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="n"/>
       <c r="K33" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6526,7 +7342,7 @@
           <t>The cart row displays an unmasked "₹ [rate]" input box, exposing commercial raw material prices to floor storekeepers and allowing them to overwrite master item pricing upon receipt.</t>
         </is>
       </c>
-      <c r="J34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="n"/>
       <c r="K34" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6592,7 +7408,7 @@
           <t>The QC role is completely denied access to GRN and PO (`grn.read` and `po.read` are missing from the QC permission matrix). QC inspectors cannot verify incoming raw materials at all.</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="n"/>
       <c r="K35" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6603,7 +7419,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M35" s="3" t="inlineStr"/>
+      <c r="M35" s="3" t="n"/>
       <c r="N35" s="3" t="n"/>
       <c r="O35" s="3" t="n"/>
     </row>
@@ -6655,7 +7471,7 @@
           <t>The server action throws a 403 Forbidden error because `commitIssue` strictly requires `store.write`, which is granted only to `STORE_GUY`, `ADMIN`, and `OWNER`. Supervisors are completely blocked from issuing materials to the floor.</t>
         </is>
       </c>
-      <c r="J36" s="3" t="inlineStr"/>
+      <c r="J36" s="3" t="n"/>
       <c r="K36" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6666,7 +7482,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M36" s="3" t="inlineStr"/>
+      <c r="M36" s="3" t="n"/>
       <c r="N36" s="3" t="n"/>
       <c r="O36" s="3" t="n"/>
     </row>
@@ -6718,7 +7534,7 @@
           <t>Machine field is blank/unselected and lists all machines in the factory. The system completely ignores existing records in `MisMachineAllocation`.</t>
         </is>
       </c>
-      <c r="J37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="n"/>
       <c r="K37" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6784,7 +7600,7 @@
           <t>Both logs are saved simultaneously without any conflict check against `MisMachineAllocation` or active running logs, causing double-booked machine data and invalid capacity reporting.</t>
         </is>
       </c>
-      <c r="J38" s="3" t="inlineStr"/>
+      <c r="J38" s="3" t="n"/>
       <c r="K38" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6795,7 +7611,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M38" s="3" t="inlineStr"/>
+      <c r="M38" s="3" t="n"/>
       <c r="N38" s="3" t="n"/>
       <c r="O38" s="3" t="n"/>
     </row>
@@ -6846,7 +7662,7 @@
           <t>The machine board still shows "Folder Gluer 01" as unallocated and idle. Production run creation never syncs or updates the machine board.</t>
         </is>
       </c>
-      <c r="J39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="n"/>
       <c r="K39" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6857,7 +7673,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M39" s="3" t="inlineStr"/>
+      <c r="M39" s="3" t="n"/>
       <c r="N39" s="3" t="n"/>
       <c r="O39" s="3" t="n"/>
     </row>
@@ -6909,7 +7725,7 @@
           <t>The allocation remains open indefinitely or until the raw `durationHours` expire on the clock, leaving machines locked as busy even after physical production finishes early.</t>
         </is>
       </c>
-      <c r="J40" s="3" t="inlineStr"/>
+      <c r="J40" s="3" t="n"/>
       <c r="K40" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -6976,7 +7792,7 @@
           <t>Machine field is empty and shows a generic dropdown of all factory machines (e.g., Slitters, Die Cutters, Gluers). An operator can mistakenly pick any random machine.</t>
         </is>
       </c>
-      <c r="J41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="n"/>
       <c r="K41" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7043,7 +7859,7 @@
           <t>The machine stays locked as "BUSY" on `/mis/machine-board` for the full 4 hours unless the Supervisor manually visits `/mis/machine-board` and clicks "Release".</t>
         </is>
       </c>
-      <c r="J42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="n"/>
       <c r="K42" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7109,7 +7925,7 @@
           <t>"Slitter 02" appears completely idle/free with 0% utilization because production logging does not create or sync with `MisMachineAllocation`.</t>
         </is>
       </c>
-      <c r="J43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="n"/>
       <c r="K43" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7120,7 +7936,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M43" s="3" t="inlineStr"/>
+      <c r="M43" s="3" t="n"/>
       <c r="N43" s="3" t="n"/>
       <c r="O43" s="3" t="n"/>
     </row>
@@ -7172,7 +7988,7 @@
           <t>No versioning exists. Reprinting does not increment version, no approval state is tracked before printing, and file naming format is completely unmanaged.</t>
         </is>
       </c>
-      <c r="J44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="n"/>
       <c r="K44" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7183,7 +7999,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M44" s="3" t="inlineStr"/>
+      <c r="M44" s="3" t="n"/>
       <c r="N44" s="3" t="n"/>
       <c r="O44" s="3" t="n"/>
     </row>
@@ -7234,7 +8050,7 @@
           <t>Worker assignment only displays a soft, ignorable warning (`confirmOverlapFor`), allowing multiple supervisors to simultaneously claim the same worker and corrupting section-wise manpower cost calculation.</t>
         </is>
       </c>
-      <c r="J45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="n"/>
       <c r="K45" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7245,7 +8061,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M45" s="3" t="inlineStr"/>
+      <c r="M45" s="3" t="n"/>
       <c r="N45" s="3" t="n"/>
       <c r="O45" s="3" t="n"/>
     </row>
@@ -7296,7 +8112,7 @@
           <t>There is no field to capture Makeready time in the UI or backend database schema (`qtyProduced`, `qtyWaste`, `unit`, `notes` only). Machine setup idle hours are lost from uptime reports.</t>
         </is>
       </c>
-      <c r="J46" s="3" t="inlineStr"/>
+      <c r="J46" s="3" t="n"/>
       <c r="K46" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7307,7 +8123,7 @@
           <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
         </is>
       </c>
-      <c r="M46" s="3" t="inlineStr"/>
+      <c r="M46" s="3" t="n"/>
       <c r="N46" s="3" t="n"/>
       <c r="O46" s="3" t="n"/>
     </row>
@@ -7359,7 +8175,7 @@
           <t>`DeviceHealthViewModel.retrySyncNow()` only triggers `PunchFlushScheduler.schedule(...)` (WorkManager punch-queue flush). It never calls `RosterRepository.sync()`. The employee roster remains completely stale, new employees/shifts are not pulled, and the cache age does not update.</t>
         </is>
       </c>
-      <c r="J47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="n"/>
       <c r="K47" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7426,7 +8242,7 @@
           <t>The app calculates `nextKindFor` exclusively from local SQLite `punch_state`, seeing the last local direction as "IN". The confirmation card hardcodes the green button to `"→ Clock out"`. There is no toggle or override option—the employee is forced to either clock OUT at shift start or tap "Not this person" and be completely locked out from clocking in.</t>
         </is>
       </c>
-      <c r="J48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="n"/>
       <c r="K48" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7493,7 +8309,7 @@
           <t>`observeClockedInCount()` runs `@Query("SELECT COUNT(*) FROM punch_state WHERE lastDirection = 'IN'")`. Because `punch_state` is never filtered by date or reset at the daily boundary, any employee who ever clocked IN on this tablet and did not clock OUT on this exact tablet remains counted as "clocked in today" indefinitely, causing the counter to permanently over-count.</t>
         </is>
       </c>
-      <c r="J49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="n"/>
       <c r="K49" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7560,7 +8376,7 @@
           <t>Android Room queries the entire `employees` table including all image byte arrays into a single SQLite `CursorWindow` (limited to 2MB–4MB in Android). Once the collective photo payloads exceed the window limit, Android throws `android.database.CursorWindowAllocationException: Row too big to fit in CursorWindow`, crashing the app process.</t>
         </is>
       </c>
-      <c r="J50" s="3" t="inlineStr"/>
+      <c r="J50" s="3" t="n"/>
       <c r="K50" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7627,7 +8443,7 @@
           <t>`RosterRepository.sync()` only invokes `credentialStore.wipe()` and `employeeDao.deleteAll()`. It leaves `active_shifts`, `punch_state`, and `rosterPreferences` intact in SQLite. Furthermore, if `/api/mis/kiosk/punch` receives a `REVOKED` response, `PunchRepository` does not check `wipe == true` and instead returns `RetryNeeded`, causing WorkManager to repeatedly retry flush requests for a retired tablet.</t>
         </is>
       </c>
-      <c r="J51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="n"/>
       <c r="K51" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7693,7 +8509,7 @@
           <t>`QrScannerView` hardcodes `CameraSelector.DEFAULT_BACK_CAMERA`. CameraX fails with `IllegalArgumentException: No camera available for CameraSelector.DEFAULT_BACK_CAMERA`. The exception is caught and logged, leaving the user staring at a black, non-functional scanner preview with no error indication or front-camera fallback.</t>
         </is>
       </c>
-      <c r="J52" s="3" t="inlineStr"/>
+      <c r="J52" s="3" t="n"/>
       <c r="K52" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7760,7 +8576,7 @@
           <t>`MainActivity` initializes `var paired by rememberSaveable { mutableStateOf(false) }`. Because it defaults to `false`, `PairingScreen` renders on screen for a frame until `PairingViewModel` initializes, confirms `activeDevice != null`, and triggers the `onPaired` callback, causing an abrupt visible flash of the pairing UI on every cold start.</t>
         </is>
       </c>
-      <c r="J53" s="3" t="inlineStr"/>
+      <c r="J53" s="3" t="n"/>
       <c r="K53" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7826,7 +8642,7 @@
           <t>`startLockTask()` is called directly inside `onResume()` without a `try-catch` block. On devices where lock task mode is blocked by system policy, calling this method throws an unhandled `SecurityException` or `IllegalArgumentException`, crashing the app immediately upon resume.</t>
         </is>
       </c>
-      <c r="J54" s="3" t="inlineStr"/>
+      <c r="J54" s="3" t="n"/>
       <c r="K54" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7893,7 +8709,7 @@
           <t>`PunchViewModel` collects the updated shifts, detects that the selected shift is missing, and clears `_selectedShift.value = null`. This causes `PunchScreen`'s shift gate to trigger abruptly, kicking the operator out of the idle/scanner screen and throwing them back to `ShiftSelectionScreen` mid-shift with no warning. (Additionally, an operator cannot intentionally switch shifts during duty without ending their shift completely and re-signing in).</t>
         </is>
       </c>
-      <c r="J55" s="3" t="inlineStr"/>
+      <c r="J55" s="3" t="n"/>
       <c r="K55" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -7961,7 +8777,7 @@
           <t>The on-screen soft keyboard occupies more than 60% of the screen height in landscape mode. Because `ManualEntryContent` uses a non-scrollable `Column` (`Modifier.fillMaxSize()`), the employee card and the green Confirm button are pushed completely below the visible screen fold, making it impossible to tap Confirm without first closing the keyboard.</t>
         </is>
       </c>
-      <c r="J56" s="3" t="inlineStr"/>
+      <c r="J56" s="3" t="n"/>
       <c r="K56" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
@@ -8028,7 +8844,7 @@
           <t>With `allowBackup="true"`, Android Cloud Backup uploads encrypted shared preferences and Room database files. Restoring to a different device causes Android Keystore decryption crashes (due to mismatched hardware master keys) or results in duplicate devices operating simultaneously with cloned tokens.</t>
         </is>
       </c>
-      <c r="J57" s="3" t="inlineStr"/>
+      <c r="J57" s="3" t="n"/>
       <c r="K57" s="3" t="inlineStr">
         <is>
           <t>round 2</t>

</xml_diff>

<commit_message>
R2 batch 3: leave pay toggle, document version snapshots, searchable item selects, tester docs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/MIS_TESTER_TRACKER.xlsx
+++ b/docs/qa/MIS_TESTER_TRACKER.xlsx
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H168"/>
+  <dimension ref="A1:H181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6888,6 +6888,448 @@
       </c>
       <c r="G168" s="3" t="n"/>
       <c r="H168" s="3" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>R2-102: Settings &gt; Leave pay: see every leave type (CL, SL, EL, LWP, Other)</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>All start Unpaid; Owner can toggle each to Paid; change is audited and history kept</t>
+        </is>
+      </c>
+      <c r="F169" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G169" s="3" t="n"/>
+      <c r="H169" s="3" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t>15.2</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="inlineStr">
+        <is>
+          <t>R2-102: Approve a CL leave for a daily worker; open payroll for that month</t>
+        </is>
+      </c>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>Payroll basic does not change while CL is Unpaid</t>
+        </is>
+      </c>
+      <c r="F170" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G170" s="3" t="n"/>
+      <c r="H170" s="3" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>15.3</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>R2-102: Set CL to Paid in Settings &gt; Leave pay; recheck the open month payroll</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>Basic rises by exactly one day rate for the approved CL day</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G171" s="3" t="n"/>
+      <c r="H171" s="3" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>15.4</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>R2-102: Flip CL back to Unpaid</t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="inlineStr">
+        <is>
+          <t>Payroll basic drops back by one day rate</t>
+        </is>
+      </c>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G172" s="3" t="n"/>
+      <c r="H172" s="3" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>R2-102: Toggle a leave type, then view a closed (past) month payroll</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
+          <t>Closed month figures are unchanged</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G173" s="3" t="n"/>
+      <c r="H173" s="3" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>15.6</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>R2-102: Open Settings &gt; Leave pay and try to change a type</t>
+        </is>
+      </c>
+      <c r="E174" s="3" t="inlineStr">
+        <is>
+          <t>Refused with 403; Admin cannot change</t>
+        </is>
+      </c>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G174" s="3" t="n"/>
+      <c r="H174" s="3" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>15.7</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>R2-46: Approve COA/job card V1 (different user from preparer); change a QC check; reprint</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>Page and file name (_V1) unchanged; content still the frozen V1</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G175" s="3" t="n"/>
+      <c r="H175" s="3" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>15.8</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>R2-46: Click 'Update to latest' (Admin or Owner)</t>
+        </is>
+      </c>
+      <c r="E176" s="3" t="inlineStr">
+        <is>
+          <t>V2 created as PREPARED; needs a different approver than the preparer</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G176" s="3" t="n"/>
+      <c r="H176" s="3" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t>15.9</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>R2-46: Open the document with ?v=1</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="inlineStr">
+        <is>
+          <t>Older V1 snapshot is viewable</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G177" s="3" t="n"/>
+      <c r="H177" s="3" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>15.10</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="inlineStr">
+        <is>
+          <t>R2-46: Open a legacy approved COA/job card (approved before this release)</t>
+        </is>
+      </c>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>Prints live data with a 'No snapshot' note</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G178" s="3" t="n"/>
+      <c r="H178" s="3" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>15.11</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>R2-82: Items &gt; Add: type in Unit, GSM, Size, Substrate, Coating</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="inlineStr">
+        <is>
+          <t>Each is a searchable dropdown that filters as you type; '+ Add new' available inline for Admin</t>
+        </is>
+      </c>
+      <c r="F179" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G179" s="3" t="n"/>
+      <c r="H179" s="3" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>15.12</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="inlineStr">
+        <is>
+          <t>R2-82: Open the same item dropdowns</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>Options listed and searchable; no '+ Add new'</t>
+        </is>
+      </c>
+      <c r="F180" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G180" s="3" t="n"/>
+      <c r="H180" s="3" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t>15.13</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>15. Round 2 — Batch 3 (release 2026-10-20) — re-test only this</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>STORE_GUY</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>R2-68/78/105 camera scanning (REAL Android Chrome device only): store issue cart Scan button; receive cart Scan; kiosk Scan with camera</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>Camera scans the barcode/employee; typed entry fallback works. Not testable on desktop or emulator</t>
+        </is>
+      </c>
+      <c r="F181" s="3" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="G181" s="3" t="n"/>
+      <c r="H181" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
@@ -6917,7 +7359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O113"/>
+  <dimension ref="A1:O112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8945,7 +9387,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>Deferred: needs schema/product input (docs/specs/00-README.md)</t>
+          <t>Blank row in the tester sheet (no title/steps); nothing to fix. Please delete or fill in if a finding was intended.</t>
         </is>
       </c>
       <c r="M27" s="3" t="n"/>
@@ -10178,12 +10620,12 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Approved COA/job-card versions are frozen snapshots; Admin/Owner get Update to latest which issues the next version for approval; older versions viewable via ?v=N. Legacy approved rows print live with a No snapshot note.</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="N44" s="3" t="inlineStr">
@@ -11172,84 +11614,84 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Bug ID</t>
+          <t>R2-62</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Fixed - Ready to Retest</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Severity</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Role / screen</t>
+          <t>Store Guy — Store Issue Screen (/mis/store/issue)</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Stock issue can be confirmed with no Order and no Department ("General issue" + "Not recorded"), creating untraceable stock outflow.</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t>1. Log in as Store Guy and navigate to Store Issue (/mis/store/issue). 2. Under "Against an order", leave "General issue" selected. 3. Under "To which department", leave "Not recorded" selected. 4. Search and add any inventory item with a valid quantity. 5. Click "Confirm issue".</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>Expected</t>
+          <t>Material issued out of the factory store must require at least an Order Number or a Department/Cost Center to maintain consumption accountability.</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Actual</t>
+          <t>The issue is successfully committed with orderId: null and departmentId: null. Stock is permanently deducted from inventory with zero attribution, creating untracked factory shrinkage.</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>round 2</t>
         </is>
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>Fix notes</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N58" s="3" t="inlineStr">
         <is>
-          <t>Retest by tester</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="O58" s="3" t="inlineStr">
         <is>
-          <t>Tester comment</t>
+          <t>Fail. Confirmed reproducible in commitIssue (src/server/mis/store.ts#L457-L490). When meta.orderId and meta.departmentId are omitted, the function resolves both to null and commits the transaction without throwing a validation error, creating untracked factory stock deductions.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>R2-62</t>
+          <t>R2-63</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -11264,32 +11706,32 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Blocker</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Store Guy — Store Issue Screen (/mis/store/issue)</t>
+          <t>Store Guy / Admin — Store Master Screen (/mis/store)</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Stock issue can be confirmed with no Order and no Department ("General issue" + "Not recorded"), creating untraceable stock outflow.</t>
+          <t>Inline "OUT" slide-over executes storeOutAction without order or department, bypassing Order Earmarks and breaking Traceability.</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as Store Guy and navigate to Store Issue (/mis/store/issue). 2. Under "Against an order", leave "General issue" selected. 3. Under "To which department", leave "Not recorded" selected. 4. Search and add any inventory item with a valid quantity. 5. Click "Confirm issue".</t>
+          <t>1. Navigate to Store Items (/mis/store). 2. Click the "OUT" button next to any raw material item. 3. Enter a valid quantity and optional reference notes in the slide-over. 4. Click "Issue Stock". 5. Check /mis/traceability and /mis/orders/[orderId] for this material.</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>Material issued out of the factory store must require at least an Order Number or a Department/Cost Center to maintain consumption accountability.</t>
+          <t>Issuing raw materials from the Store master screen should either redirect to /mis/store/issue or prompt for an Order/Department so that order allocations and batch traceability are updated.</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>The issue is successfully committed with orderId: null and departmentId: null. Stock is permanently deducted from inventory with zero attribution, creating untracked factory shrinkage.</t>
+          <t>The inline slide-over executes storeOutAction, which takes only itemId, quantity, and referenceNo. It writes sourceId: null in MisInventoryLedger, completely bypassing MisOrderStockAllocation and rendering the material invisible in /mis/traceability.</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
@@ -11319,19 +11761,19 @@
       </c>
       <c r="O59" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in commitIssue (src/server/mis/store.ts#L457-L490). When meta.orderId and meta.departmentId are omitted, the function resolves both to null and commits the transaction without throwing a validation error, creating untracked factory stock deductions.</t>
+          <t>Fail. Confirmed reproducible in createStoreOut (src/server/mis/store.ts#L416-L442) and store-item-screen.tsx#L154. storeOutAction commits a stock deduction with hardcoded sourceId: null in misInventoryLedger without order or department binding, bypassing allocationShortfalls and breaking order traceability.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>R2-63</t>
+          <t>R2-64</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Enhancement</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -11341,37 +11783,37 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Blocker</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Store Guy / Admin — Store Master Screen (/mis/store)</t>
+          <t>All Roles (Store Guy, Admin, Owner) — Desktop Sidebar Navigation (/mis/*)</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Inline "OUT" slide-over executes storeOutAction without order or department, bypassing Order Earmarks and breaking Traceability.</t>
+          <t>Desktop sidebar has only a single flat link to /mis/store; Dashboard, Goods Issue, Receipts, and Transaction Logs are missing from navigation.</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>1. Navigate to Store Items (/mis/store). 2. Click the "OUT" button next to any raw material item. 3. Enter a valid quantity and optional reference notes in the slide-over. 4. Click "Issue Stock". 5. Check /mis/traceability and /mis/orders/[orderId] for this material.</t>
+          <t>1. Log in on desktop as Store Guy, Admin, or Owner. 2. Look at the desktop sidebar navigation under the unlabelled section. 3. Observe that only a single link /mis/store is present. 4. Attempt to navigate from the sidebar to Store Dashboard (/mis/store/dashboard), Goods Issue (/mis/store/issue), or Transaction Logs (/mis/store/transactions).</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>Issuing raw materials from the Store master screen should either redirect to /mis/store/issue or prompt for an Order/Department so that order allocations and batch traceability are updated.</t>
+          <t>As per ERP standards and operational workflows, the Store section should have structured sub-navigation items: Dashboard (/mis/store/dashboard), Store Items (/mis/store), Goods Issue (/mis/store/issue), Goods Receipt (/mis/store/receive), Material Requests (/mis/store/requests), Physical Count (/mis/store/count), and Transaction Logs (/mis/store/transactions).</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>The inline slide-over executes storeOutAction, which takes only itemId, quantity, and referenceNo. It writes sourceId: null in MisInventoryLedger, completely bypassing MisOrderStockAllocation and rendering the material invisible in /mis/traceability.</t>
+          <t>The desktop sidebar contains only a single flat link /mis/store (opening the raw items table). Seven core store workflows are completely orphaned from the sidebar menu and can only be reached via manual URL entry or home tiles.</t>
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
@@ -11381,12 +11823,12 @@
       </c>
       <c r="L60" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M60" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N60" s="3" t="inlineStr">
@@ -11396,19 +11838,19 @@
       </c>
       <c r="O60" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in createStoreOut (src/server/mis/store.ts#L416-L442) and store-item-screen.tsx#L154. storeOutAction commits a stock deduction with hardcoded sourceId: null in misInventoryLedger without order or department binding, bypassing allocationShortfalls and breaking order traceability.</t>
+          <t>Fail. Confirmed reproducible in NAV (src/server/mis/navigation.ts#L48) and groupDesktopNav (src/lib/mis/desktop-nav.ts#L32-L46). The desktop navigation registry only exposes a single flat /mis/store item. Sub-workflows (dashboard, issue, receive, requests, transactions) have no sidebar entries and are accessible only via home tiles or manual URL.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>R2-64</t>
+          <t>R2-65</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -11418,37 +11860,37 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>All Roles (Store Guy, Admin, Owner) — Desktop Sidebar Navigation (/mis/*)</t>
+          <t>Supervisor — Material Request Screen (/mis/store/requests/new)</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Desktop sidebar has only a single flat link to /mis/store; Dashboard, Goods Issue, Receipts, and Transaction Logs are missing from navigation.</t>
+          <t>Post-submission UI glitch: Cart form and selected chips remain interactive below the green confirmation card.</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>1. Log in on desktop as Store Guy, Admin, or Owner. 2. Look at the desktop sidebar navigation under the unlabelled section. 3. Observe that only a single link /mis/store is present. 4. Attempt to navigate from the sidebar to Store Dashboard (/mis/store/dashboard), Goods Issue (/mis/store/issue), or Transaction Logs (/mis/store/transactions).</t>
+          <t>1. From Supervisor Home, click "Request material from the store" (/mis/store/requests/new). 2. Choose a department (e.g. Printing). 3. Search and add 2 items to the cart. 4. Click "Send request". 5. Observe the screen after submission.</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>As per ERP standards and operational workflows, the Store section should have structured sub-navigation items: Dashboard (/mis/store/dashboard), Store Items (/mis/store), Goods Issue (/mis/store/issue), Goods Receipt (/mis/store/receive), Material Requests (/mis/store/requests), Physical Count (/mis/store/count), and Transaction Logs (/mis/store/transactions).</t>
+          <t>The green card "MRN-... is waiting for the Store" should appear, and the form should cleanly transition to a confirmation view with an option to "Create Another Request" or return Home.</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>The desktop sidebar contains only a single flat link /mis/store (opening the raw items table). Seven core store workflows are completely orphaned from the sidebar menu and can only be reached via manual URL entry or home tiles.</t>
+          <t>The green &lt;OkCard&gt; appears at the top, but the &lt;ItemCart&gt; search bar, department chips, and order chips remain visible and interactive directly below it, leading users to believe the request is still pending submission.</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
@@ -11458,12 +11900,12 @@
       </c>
       <c r="L61" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M61" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N61" s="3" t="inlineStr">
@@ -11473,19 +11915,19 @@
       </c>
       <c r="O61" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in NAV (src/server/mis/navigation.ts#L48) and groupDesktopNav (src/lib/mis/desktop-nav.ts#L32-L46). The desktop navigation registry only exposes a single flat /mis/store item. Sub-workflows (dashboard, issue, receive, requests, transactions) have no sidebar entries and are accessible only via home tiles or manual URL.</t>
+          <t>Fail. Confirmed reproducible in RequestScreen (src/components/mis/store/request-screen.tsx#L53-L75). When done state is set, &lt;OkCard&gt; renders at the top of the stack, but &lt;ItemCart&gt; and the department/order selector cards remain rendered and interactive directly beneath it instead of being hidden or unmounted.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>R2-65</t>
+          <t>R2-66</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Enhancement</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -11500,27 +11942,27 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Supervisor — Material Request Screen (/mis/store/requests/new)</t>
+          <t>Store Guy — Store Issue Screen (/mis/store/issue)</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Post-submission UI glitch: Cart form and selected chips remain interactive below the green confirmation card.</t>
+          <t>Cart displays stale stock balance without real-time updates, leading to silent commit failure when another terminal issues stock.</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>1. From Supervisor Home, click "Request material from the store" (/mis/store/requests/new). 2. Choose a department (e.g. Printing). 3. Search and add 2 items to the cart. 4. Click "Send request". 5. Observe the screen after submission.</t>
+          <t>1. Open /mis/store/issue on Terminal A and search for an item with 10 units in stock. 2. On Terminal B, issue 5 units of the same item. 3. On Terminal A, enter quantity 10 (still displayed as available on screen). 4. Click "Confirm issue".</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>The green card "MRN-... is waiting for the Store" should appear, and the form should cleanly transition to a confirmation view with an option to "Create Another Request" or return Home.</t>
+          <t>The cart should display real-time available stock or alert the user before confirmation that available stock has changed.</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>The green &lt;OkCard&gt; appears at the top, but the &lt;ItemCart&gt; search bar, department chips, and order chips remain visible and interactive directly below it, leading users to believe the request is still pending submission.</t>
+          <t>Terminal A allows typing 10 with no warning. Upon clicking "Confirm issue", the entire cart fails with a red error card: "Cannot issue more than the stock balance (5 available)", requiring the user to re-evaluate and re-type the line.</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
@@ -11535,12 +11977,12 @@
       </c>
       <c r="L62" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N62" s="3" t="inlineStr">
@@ -11550,14 +11992,14 @@
       </c>
       <c r="O62" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in RequestScreen (src/components/mis/store/request-screen.tsx#L53-L75). When done state is set, &lt;OkCard&gt; renders at the top of the stack, but &lt;ItemCart&gt; and the department/order selector cards remain rendered and interactive directly beneath it instead of being hidden or unmounted.</t>
+          <t>Fail. Confirmed in IssueScreen (src/components/mis/store/issue-screen.tsx#L16-L23). Available stock quantities are passed as static server component props at initial page load without real-time socket subscription or focus-triggered balance revalidation, leading to optimistic concurrency rejections at commit time.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>R2-66</t>
+          <t>R2-67</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -11577,27 +12019,27 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Store Guy — Store Issue Screen (/mis/store/issue)</t>
+          <t>Supervisor — Material Request Flow (/mis/store/requests/*)</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Cart displays stale stock balance without real-time updates, leading to silent commit failure when another terminal issues stock.</t>
+          <t>No push notification or status alert sent to Supervisor when Store Guy decides (approves/rejects) an MRN.</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/store/issue on Terminal A and search for an item with 10 units in stock. 2. On Terminal B, issue 5 units of the same item. 3. On Terminal A, enter quantity 10 (still displayed as available on screen). 4. Click "Confirm issue".</t>
+          <t>1. Supervisor submits a Material Request from /mis/store/requests/new. 2. Store Guy opens /mis/store/requests/[id] and either approves with reduced quantity or rejects with a reason note. 3. Observe Supervisor's Home screen and Notification Bell.</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>The cart should display real-time available stock or alert the user before confirmation that available stock has changed.</t>
+          <t>Supervisor should receive an in-app alert or notification bell counter update informing them that MRN-XXXX has been approved or rejected.</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Terminal A allows typing 10 with no warning. Upon clicking "Confirm issue", the entire cart fails with a red error card: "Cannot issue more than the stock balance (5 available)", requiring the user to re-evaluate and re-type the line.</t>
+          <t>No notification or bell ping is sent to the Supervisor. The Supervisor has to manually remember the MRN number and open the URL to see if materials are ready for pickup.</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
@@ -11627,14 +12069,14 @@
       </c>
       <c r="O63" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed in IssueScreen (src/components/mis/store/issue-screen.tsx#L16-L23). Available stock quantities are passed as static server component props at initial page load without real-time socket subscription or focus-triggered balance revalidation, leading to optimistic concurrency rejections at commit time.</t>
+          <t>Fail. Confirmed in rejectMaterialRequest and fulfillMaterialRequest (src/server/mis/material-request.ts#L170-L215). While createMaterialRequest dispatches notification to STORE_GUY, store decision actions lack notification triggers to inform the requesting supervisor of approval or rejection.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>R2-67</t>
+          <t>R2-68</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -11654,32 +12096,32 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Supervisor — Material Request Flow (/mis/store/requests/*)</t>
+          <t>Store Guy — Goods Issue Screen (/mis/store/issue)</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>No push notification or status alert sent to Supervisor when Store Guy decides (approves/rejects) an MRN.</t>
+          <t>Lack of Barcode / QR Code scanning input for fast physical warehouse picking.</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>1. Supervisor submits a Material Request from /mis/store/requests/new. 2. Store Guy opens /mis/store/requests/[id] and either approves with reduced quantity or rejects with a reason note. 3. Observe Supervisor's Home screen and Notification Bell.</t>
+          <t>1. Open /mis/store/issue on a mobile/tablet warehouse scanner. 2. Attempt to scan physical item barcode or GRN batch QR code to add line to cart.</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>Supervisor should receive an in-app alert or notification bell counter update informing them that MRN-XXXX has been approved or rejected.</t>
+          <t>Warehouse goods issue should provide a camera/hardware barcode scan button to immediately look up and add items by SKU/Code.</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>No notification or bell ping is sent to the Supervisor. The Supervisor has to manually remember the MRN number and open the URL to see if materials are ready for pickup.</t>
+          <t>Only manual text typing in the search input is supported. Storekeepers must manually type item codes on a virtual keyboard for every item dispatched.</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>Mobile / Tablet</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
@@ -11689,12 +12131,12 @@
       </c>
       <c r="L64" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Camera scanning built; needs a real device (Chrome on Android) — tester to verify; typed entry works everywhere.</t>
         </is>
       </c>
       <c r="M64" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="N64" s="3" t="inlineStr">
@@ -11704,19 +12146,19 @@
       </c>
       <c r="O64" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed in rejectMaterialRequest and fulfillMaterialRequest (src/server/mis/material-request.ts#L170-L215). While createMaterialRequest dispatches notification to STORE_GUY, store decision actions lack notification triggers to inform the requesting supervisor of approval or rejection.</t>
+          <t>Fail. Confirmed in ItemCart (src/components/mis/store/item-cart.tsx#L140-L165). Search bar relies entirely on text typing or external USB HID wedge scanners. There is no camera barcode/QR scanner integration for mobile/tablet warehouse pickers.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>R2-68</t>
+          <t>R2-69</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -11726,37 +12168,37 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Store Guy — Goods Issue Screen (/mis/store/issue)</t>
+          <t>Admin / Purchase Officer — Purchase Orders Screen (/mis/po)</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Lack of Barcode / QR Code scanning input for fast physical warehouse picking.</t>
+          <t>Purchase Order can be created without selecting a Supplier (no mandatory supplier validation on PO creation).</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/store/issue on a mobile/tablet warehouse scanner. 2. Attempt to scan physical item barcode or GRN batch QR code to add line to cart.</t>
+          <t>1. Log in as Admin or Owner and navigate to Purchase Orders (/mis/po). 2. Click on "+ New PO" to open the creation slide-over modal. 3. Leave the Supplier dropdown on the default "— Select supplier —" (unselected). 4. Select Purpose as "Buffer stock — no BOM" (or select an approved BOM reference). 5. Click Create/Submit to create the Purchase Order.</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>Warehouse goods issue should provide a camera/hardware barcode scan button to immediately look up and add items by SKU/Code.</t>
+          <t>The Supplier field must be mandatory. If no supplier is selected, the form should display a client-side validation error ("Please select a supplier") and the backend should reject creation, as a Purchase Order is a commercial contract that cannot exist without a vendor.</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Only manual text typing in the search input is supported. Storekeepers must manually type item codes on a virtual keyboard for every item dispatched.</t>
+          <t>The PO is created successfully with supplierId: null. The system generates an official PO number (e.g. PO-202610-00018), saves it to mis_purchase_orders, and displays it in the table with Supplier as "—".</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>Mobile / Tablet</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
@@ -11766,12 +12208,12 @@
       </c>
       <c r="L65" s="3" t="inlineStr">
         <is>
-          <t>Camera scanning built; needs real-device test (Chrome/Android) — typed fallback works everywhere</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M65" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N65" s="3" t="inlineStr">
@@ -11781,14 +12223,14 @@
       </c>
       <c r="O65" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed in ItemCart (src/components/mis/store/item-cart.tsx#L140-L165). Search bar relies entirely on text typing or external USB HID wedge scanners. There is no camera barcode/QR scanner integration for mobile/tablet warehouse pickers.</t>
+          <t>Fail. Confirmed reproducible in handleCreate (src/components/mis/po/po-list-screen.tsx#L55-L60) and createPO (src/server/mis/po.ts#L45-L55). Neither client form submission nor backend createPO enforces supplierId existence, permitting orphan PO creation with supplierId: null.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>R2-69</t>
+          <t>R2-70</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -11808,27 +12250,27 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Admin / Purchase Officer — Purchase Orders Screen (/mis/po)</t>
+          <t>Admin / Planner — BOM Detail / Edit Screen (/mis/bom/[orderId]?view=edit)</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Purchase Order can be created without selecting a Supplier (no mandatory supplier validation on PO creation).</t>
+          <t>Stage name in BOM builder is a free-text input instead of a dropdown populated from Master Processes (MisProcess).</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as Admin or Owner and navigate to Purchase Orders (/mis/po). 2. Click on "+ New PO" to open the creation slide-over modal. 3. Leave the Supplier dropdown on the default "— Select supplier —" (unselected). 4. Select Purpose as "Buffer stock — no BOM" (or select an approved BOM reference). 5. Click Create/Submit to create the Purchase Order.</t>
+          <t>1. Log in as Admin or Owner and navigate to an Order's BOM in edit view (/mis/bom/[orderId]?view=edit). 2. Click on "+ Add Stage" to open the slide-over modal (or click "Edit" on an existing stage). 3. Observe the input field provided for Stage Name.</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>The Supplier field must be mandatory. If no supplier is selected, the form should display a client-side validation error ("Please select a supplier") and the backend should reject creation, as a Purchase Order is a commercial contract that cannot exist without a vendor.</t>
+          <t>Stage Name should be a standardized dropdown (&lt;Select&gt;) populated from the Master Process table (MisProcess). Selecting a process should automatically set stageName and link processId on MisBomStage so production machines, line clearance, and QC templates can link to the stage.</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>The PO is created successfully with supplierId: null. The system generates an official PO number (e.g. PO-202610-00018), saves it to mis_purchase_orders, and displays it in the table with Supplier as "—".</t>
+          <t>Stage Name is rendered as a plain text input (&lt;Input label="Stage Name" /&gt;). Users must manually type stage names as free text. As a result, processId is left null in mis_bom_stages, disconnecting BOM stages from master process routing, machine allocation, and stage-wise QC checklists.</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
@@ -11858,14 +12300,14 @@
       </c>
       <c r="O66" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in handleCreate (src/components/mis/po/po-list-screen.tsx#L55-L60) and createPO (src/server/mis/po.ts#L45-L55). Neither client form submission nor backend createPO enforces supplierId existence, permitting orphan PO creation with supplierId: null.</t>
+          <t>Fail. Confirmed reproducible in BomScreen (src/components/mis/bom/bom-screen.tsx#L162-L182). Add Stage and Edit Stage slide-overs render free-text &lt;Input label="Stage Name"&gt; instead of a &lt;Select&gt; dropdown sourcing from MisProcess, leaving processId null in mis_bom_stages and disconnecting stages from master routing.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>R2-70</t>
+          <t>R2-71</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -11885,27 +12327,27 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Admin / Planner — BOM Detail / Edit Screen (/mis/bom/[orderId]?view=edit)</t>
+          <t>Store Guy — Goods Receipt Screen (`/mis/grn/[id]`)</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Stage name in BOM builder is a free-text input instead of a dropdown populated from Master Processes (MisProcess).</t>
+          <t>When line type is "For Specific Order", Order Reference is a free-text input instead of a dropdown of Confirmed Orders.</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as Admin or Owner and navigate to an Order's BOM in edit view (/mis/bom/[orderId]?view=edit). 2. Click on "+ Add Stage" to open the slide-over modal (or click "Edit" on an existing stage). 3. Observe the input field provided for Stage Name.</t>
+          <t>1. Log in as Store Guy and open a draft GRN (`/mis/grn/[id]`). 2. Under "Add Item", select a PO line item. 3. Change the "Type" dropdown from "General Stock" to "For Specific Order". 4. Observe the "Order Reference" input field rendered below.</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>Stage Name should be a standardized dropdown (&lt;Select&gt;) populated from the Master Process table (MisProcess). Selecting a process should automatically set stageName and link processId on MisBomStage so production machines, line clearance, and QC templates can link to the stage.</t>
+          <t>When "For Specific Order" is selected, the system must render a dropdown (`&lt;Select&gt;`) populated with active confirmed orders (status `CONFIRMED` or `IN_PRODUCTION`), displaying Order Number and Customer Name, so users can select an existing order without typing errors.</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Stage Name is rendered as a plain text input (&lt;Input label="Stage Name" /&gt;). Users must manually type stage names as free text. As a result, processId is left null in mis_bom_stages, disconnecting BOM stages from master process routing, machine allocation, and stage-wise QC checklists.</t>
+          <t>Order Reference is rendered as a plain free-text field (`&lt;Input label="Order Reference" /&gt;`). Users must manually type the order string. Any typo in the order string causes `allocateFromReceipt` to silently return `null`, so the GRN commits without creating any `MisOrderStockAllocation` earmark for the order.</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
@@ -11935,14 +12377,14 @@
       </c>
       <c r="O67" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in BomScreen (src/components/mis/bom/bom-screen.tsx#L162-L182). Add Stage and Edit Stage slide-overs render free-text &lt;Input label="Stage Name"&gt; instead of a &lt;Select&gt; dropdown sourcing from MisProcess, leaving processId null in mis_bom_stages and disconnecting stages from master routing.</t>
+          <t>Fail. Confirmed reproducible in GrnDetailScreen (src/components/mis/grn/grn-detail-screen.tsx#L254-L260). When type is 'FOR_ORDER', Order Reference is rendered as an unvalidated free-text &lt;Input&gt; rather than a &lt;Select&gt; dropdown sourcing from confirmed MisOrder records. Typos cause allocateFromReceipt (src/server/mis/grn.ts) to silently fail to find the order, skipping stock reservation.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>R2-71</t>
+          <t>R2-72</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -11962,27 +12404,27 @@
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Store Guy — Goods Receipt Screen (`/mis/grn/[id]`)</t>
+          <t>Store Guy / Owner — Goods Receipt Screen (`/mis/grn/[id]`)</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>When line type is "For Specific Order", Order Reference is a free-text input instead of a dropdown of Confirmed Orders.</t>
+          <t>Unsaved Delivery Paperwork (Invoice No, DC No, Vehicle) is silently discarded when clicking "Confirm GRN".</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as Store Guy and open a draft GRN (`/mis/grn/[id]`). 2. Under "Add Item", select a PO line item. 3. Change the "Type" dropdown from "General Stock" to "For Specific Order". 4. Observe the "Order Reference" input field rendered below.</t>
+          <t>1. Open a draft GRN (`/mis/grn/[id]`). 2. Fill in the Delivery Paperwork fields (Supplier Invoice No, DC No, LR No, Vehicle No). 3. Do NOT click the separate "Save paperwork" button. 4. Directly click "Confirm GRN" at the top right. 5. Inspect the confirmed GRN details and the 3-Way Match table on the PO.</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>When "For Specific Order" is selected, the system must render a dropdown (`&lt;Select&gt;`) populated with active confirmed orders (status `CONFIRMED` or `IN_PRODUCTION`), displaying Order Number and Customer Name, so users can select an existing order without typing errors.</t>
+          <t>Clicking "Confirm GRN" should automatically save and persist all entered paperwork fields before confirming the GRN, or warn the user that paperwork changes are unsaved.</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>Order Reference is rendered as a plain free-text field (`&lt;Input label="Order Reference" /&gt;`). Users must manually type the order string. Any typo in the order string causes `allocateFromReceipt` to silently return `null`, so the GRN commits without creating any `MisOrderStockAllocation` earmark for the order.</t>
+          <t>The "Confirm GRN" button only triggers `confirmGrnAction()`, which reads the GRN from the database where paperwork is still null. The paperwork typed in the form is silently discarded, and no `MisSupplierInvoice` is created for the 3-Way Match.</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
@@ -12012,14 +12454,14 @@
       </c>
       <c r="O68" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in GrnDetailScreen (src/components/mis/grn/grn-detail-screen.tsx#L254-L260). When type is 'FOR_ORDER', Order Reference is rendered as an unvalidated free-text &lt;Input&gt; rather than a &lt;Select&gt; dropdown sourcing from confirmed MisOrder records. Typos cause allocateFromReceipt (src/server/mis/grn.ts) to silently fail to find the order, skipping stock reservation.</t>
+          <t>Fail. Confirmed reproducible in GrnDetailScreen (src/components/mis/grn/grn-detail-screen.tsx#L125-L140). handleConfirm directly triggers confirmGrnAction(grn.id) without calling handleSaveHeader or saving dirty paperwork fields. Any typed Invoice No, DC No, or Vehicle details left unsaved are discarded, preventing MisSupplierInvoice 3-way match creation.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>R2-72</t>
+          <t>R2-73</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -12039,27 +12481,27 @@
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Store Guy / Owner — Goods Receipt Screen (`/mis/grn/[id]`)</t>
+          <t>Store Guy — Goods Receipt Screen (`/mis/grn/[id]`)</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Unsaved Delivery Paperwork (Invoice No, DC No, Vehicle) is silently discarded when clicking "Confirm GRN".</t>
+          <t>GRN can be confirmed with completely blank Delivery Paperwork (no DC Number or Invoice Number).</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>1. Open a draft GRN (`/mis/grn/[id]`). 2. Fill in the Delivery Paperwork fields (Supplier Invoice No, DC No, LR No, Vehicle No). 3. Do NOT click the separate "Save paperwork" button. 4. Directly click "Confirm GRN" at the top right. 5. Inspect the confirmed GRN details and the 3-Way Match table on the PO.</t>
+          <t>1. Create a new GRN against an approved PO (`/mis/grn`). 2. Open the draft GRN. 3. Add items with received quantities, leaving all paperwork fields (Invoice No, DC No, Vehicle No) blank. 4. Click "Confirm GRN".</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>Clicking "Confirm GRN" should automatically save and persist all entered paperwork fields before confirming the GRN, or warn the user that paperwork changes are unsaved.</t>
+          <t>A GRN represents physical delivery backed by vendor documentation. The system should require at least a Delivery Challan Number (DC No) or Supplier Invoice No before allowing confirmation.</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>The "Confirm GRN" button only triggers `confirmGrnAction()`, which reads the GRN from the database where paperwork is still null. The paperwork typed in the form is silently discarded, and no `MisSupplierInvoice` is created for the 3-Way Match.</t>
+          <t>`assertConfirmable()` only verifies item quantities and catalog mappings. The GRN confirms successfully with zero paperwork. Without a supplier invoice number, the 3-Way Match record is never generated.</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
@@ -12089,14 +12531,14 @@
       </c>
       <c r="O69" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in GrnDetailScreen (src/components/mis/grn/grn-detail-screen.tsx#L125-L140). handleConfirm directly triggers confirmGrnAction(grn.id) without calling handleSaveHeader or saving dirty paperwork fields. Any typed Invoice No, DC No, or Vehicle details left unsaved are discarded, preventing MisSupplierInvoice 3-way match creation.</t>
+          <t>Fail. Confirmed reproducible in assertConfirmable (src/server/mis/grn.ts#L363-L375). Neither assertConfirmable nor confirmGRN validates presence of delivery paperwork (dcNumber or supplierInvoiceNo), allowing goods to be booked into warehouse inventory with zero shipping document or invoice references.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>R2-73</t>
+          <t>R2-74</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -12111,32 +12553,32 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Store Guy — Goods Receipt Screen (`/mis/grn/[id]`)</t>
+          <t>Store Guy — Goods Receipt Item Modal (`/mis/grn/[id]`)</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>GRN can be confirmed with completely blank Delivery Paperwork (no DC Number or Invoice Number).</t>
+          <t>Blank DC Quantity bypasses Challan shortage arithmetic and excess delivery validation.</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>1. Create a new GRN against an approved PO (`/mis/grn`). 2. Open the draft GRN. 3. Add items with received quantities, leaving all paperwork fields (Invoice No, DC No, Vehicle No) blank. 4. Click "Confirm GRN".</t>
+          <t>1. On a draft GRN, select a PO item. 2. Leave "DC Qty" blank. 3. Enter Received Qty as 100 and Damaged Qty as 10. 4. Click "Add Item".</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>A GRN represents physical delivery backed by vendor documentation. The system should require at least a Delivery Challan Number (DC No) or Supplier Invoice No before allowing confirmation.</t>
+          <t>When receiving against a delivery challan, DC Qty should be mandatory so the system can verify that Received + Damaged &lt;= DC Qty and accurately compute Short Qty.</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>`assertConfirmable()` only verifies item quantities and catalog mappings. The GRN confirms successfully with zero paperwork. Without a supplier invoice number, the 3-Way Match record is never generated.</t>
+          <t>Leaving DC Qty blank sets `dcQuantity` to null. The validation check (`accounted &gt; dc`) in `shortQuantity()` is skipped, and `shortQuantity` returns null, disabling shortage auditing.</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
@@ -12151,12 +12593,12 @@
       </c>
       <c r="L70" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M70" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N70" s="3" t="inlineStr">
@@ -12166,14 +12608,14 @@
       </c>
       <c r="O70" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in assertConfirmable (src/server/mis/grn.ts#L363-L375). Neither assertConfirmable nor confirmGRN validates presence of delivery paperwork (dcNumber or supplierInvoiceNo), allowing goods to be booked into warehouse inventory with zero shipping document or invoice references.</t>
+          <t>Fail. Confirmed reproducible in shortQuantity (src/lib/mis/grn-match.ts#L1-L10). When dcQuantity is left blank, dc is null, causing shortQuantity to immediately return null without executing the accounted &gt; dc excess delivery guard or calculating in-transit shortage.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>R2-74</t>
+          <t>R2-75</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -12193,27 +12635,27 @@
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Store Guy — Goods Receipt Item Modal (`/mis/grn/[id]`)</t>
+          <t>Store Guy / Admin — Purchase Orders &amp; GRN Flow (`/mis/po/[id]`)</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Blank DC Quantity bypasses Challan shortage arithmetic and excess delivery validation.</t>
+          <t>100% damaged delivery leaves Purchase Order status stalled without reflecting receipt attempt.</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>1. On a draft GRN, select a PO item. 2. Leave "DC Qty" blank. 3. Enter Received Qty as 100 and Damaged Qty as 10. 4. Click "Add Item".</t>
+          <t>1. On a draft GRN, add an item with Received Qty = 0 and Damaged Qty = 50. 2. Confirm the GRN. 3. Open the linked Purchase Order (`/mis/po/[id]`).</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>When receiving against a delivery challan, DC Qty should be mandatory so the system can verify that Received + Damaged &lt;= DC Qty and accurately compute Short Qty.</t>
+          <t>The PO should reflect that a delivery took place and goods were rejected/damaged (e.g., transition to `RECEIVING` or show damaged counter).</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Leaving DC Qty blank sets `dcQuantity` to null. The validation check (`accounted &gt; dc`) in `shortQuantity()` is skipped, and `shortQuantity` returns null, disabling shortage auditing.</t>
+          <t>Because `receivedQty` is 0, `poStatusAfterReceipt()` is skipped entirely. The PO remains stuck in `APPROVED` with `receivedQuantity = 0`, leaving no indication on the PO list that the vendor attempted delivery.</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
@@ -12228,12 +12670,12 @@
       </c>
       <c r="L71" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M71" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N71" s="3" t="inlineStr">
@@ -12243,14 +12685,14 @@
       </c>
       <c r="O71" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in shortQuantity (src/lib/mis/grn-match.ts#L1-L10). When dcQuantity is left blank, dc is null, causing shortQuantity to immediately return null without executing the accounted &gt; dc excess delivery guard or calculating in-transit shortage.</t>
+          <t>Fail. Confirmed reproducible in confirmGRN (src/server/mis/grn.ts#L472-L478). poStatusAfterReceipt is guarded by [...received.values()].some((q) =&gt; q &gt; 0). If a delivery arrives with 100% damaged items (receivedQty = 0), this check evaluates to false, leaving the PO in APPROVED with receivedQuantity = 0 and no indication of receipt.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>R2-75</t>
+          <t>R2-76</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -12265,32 +12707,32 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Store Guy / Admin — Purchase Orders &amp; GRN Flow (`/mis/po/[id]`)</t>
+          <t>Store Guy / All Roles — Store Issue Screen (`/mis/store/issue`)</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>100% damaged delivery leaves Purchase Order status stalled without reflecting receipt attempt.</t>
+          <t>Server Action throws obfuscated 500 error ("An error occurred in the Server Components render…") on Confirm Issue instead of a user-friendly error message.</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>1. On a draft GRN, add an item with Received Qty = 0 and Damaged Qty = 50. 2. Confirm the GRN. 3. Open the linked Purchase Order (`/mis/po/[id]`).</t>
+          <t>1. Open Store Issue screen (`/mis/store/issue`). 2. Add an item with a valid quantity to the cart. 3. Click "Confirm issue". 4. Observe the red error banner rendered in the cart.</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>The PO should reflect that a delivery took place and goods were rejected/damaged (e.g., transition to `RECEIVING` or show damaged counter).</t>
+          <t>If the action fails due to permission boundaries, allocation shortfall, or database lock, the screen should display a clear, friendly error message (e.g., "You do not have permission to issue stock" or "Connection busy, please retry").</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>Because `receivedQty` is 0, `poStatusAfterReceipt()` is skipped entirely. The PO remains stuck in `APPROVED` with `receivedQuantity = 0`, leaving no indication on the PO list that the vendor attempted delivery.</t>
+          <t>The server action re-throws an unhandled error across the Server Component boundary, causing Next.js production build to redact it to: "An error occurred in the Server Components render. The specific message is omitted in production builds to avoid leaking sensitive details."</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
@@ -12320,19 +12762,19 @@
       </c>
       <c r="O72" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in confirmGRN (src/server/mis/grn.ts#L472-L478). poStatusAfterReceipt is guarded by [...received.values()].some((q) =&gt; q &gt; 0). If a delivery arrives with 100% damaged items (receivedQty = 0), this check evaluates to false, leaving the PO in APPROVED with receivedQuantity = 0 and no indication of receipt.</t>
+          <t>Fail. Confirmed reproducible in asResult (src/lib/mis/action-result.ts#L65-L75). asResult explicitly re-throws isForbidden(error) across the server action boundary. In Next.js production builds, uncaught server action errors are redacted to 'An error occurred in the Server Components render...', masking 403 permission refusals with a cryptic 500-style error.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>R2-76</t>
+          <t>R2-77</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Enhancement</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -12347,27 +12789,27 @@
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Store Guy / All Roles — Store Issue Screen (`/mis/store/issue`)</t>
+          <t>Store &amp; Warehouse Management (`/mis/store/issue` &amp; `/mis/store`)</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Server Action throws obfuscated 500 error ("An error occurred in the Server Components render…") on Confirm Issue instead of a user-friendly error message.</t>
+          <t>UI/UX Gap (ERP Standard): Missing 2-step Picking &amp; Staging workflow (Pick List generation ➔ Staging ➔ Floor Dispatch).</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>1. Open Store Issue screen (`/mis/store/issue`). 2. Add an item with a valid quantity to the cart. 3. Click "Confirm issue". 4. Observe the red error banner rendered in the cart.</t>
+          <t>1. Open Store Issue (`/mis/store/issue`). 2. Attempt to prepare or pick a bulk material dispatch list for a production order in advance.</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>If the action fails due to permission boundaries, allocation shortfall, or database lock, the screen should display a clear, friendly error message (e.g., "You do not have permission to issue stock" or "Connection busy, please retry").</t>
+          <t>Industry ERPs (SAP WM / Odoo Inventory) provide a two-step dispatch: 1) Generate Pick List from BOM/Job Order, 2) Warehouse picker marks items staged, 3) Final handover to machine operator deducts stock.</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>The server action re-throws an unhandled error across the Server Component boundary, causing Next.js production build to redact it to: "An error occurred in the Server Components render. The specific message is omitted in production builds to avoid leaking sensitive details."</t>
+          <t>The current screen only supports a 1-step direct debit cart. There is no intermediate "Staged / Ready for Pickup" status or printable picking slip for large packaging orders.</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
@@ -12382,12 +12824,12 @@
       </c>
       <c r="L73" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M73" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N73" s="3" t="inlineStr">
@@ -12397,14 +12839,14 @@
       </c>
       <c r="O73" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed reproducible in asResult (src/lib/mis/action-result.ts#L65-L75). asResult explicitly re-throws isForbidden(error) across the server action boundary. In Next.js production builds, uncaught server action errors are redacted to 'An error occurred in the Server Components render...', masking 403 permission refusals with a cryptic 500-style error.</t>
+          <t>Fail. Confirmed architectural gap in store issue flow (src/components/mis/store/issue-screen.tsx). The system supports only immediate 1-step direct ledger debit on cart confirm. There is no intermediate 'Staged' state, staging location tracking, or printable pick list slip for production orders.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>R2-77</t>
+          <t>R2-78</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -12424,32 +12866,32 @@
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Store &amp; Warehouse Management (`/mis/store/issue` &amp; `/mis/store`)</t>
+          <t>Store Guy / Mobile Kiosk — Goods Issue &amp; Receive Cart (`/mis/store/issue`, `/mis/store/receive`)</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>UI/UX Gap (ERP Standard): Missing 2-step Picking &amp; Staging workflow (Pick List generation ➔ Staging ➔ Floor Dispatch).</t>
+          <t>UI/UX Gap (ERP Standard): No integrated Barcode / 2D QR Code camera scanner in Item Cart for physical warehouse picking.</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>1. Open Store Issue (`/mis/store/issue`). 2. Attempt to prepare or pick a bulk material dispatch list for a production order in advance.</t>
+          <t>1. Open `/mis/store/issue` or `/mis/store/receive` on a mobile/tablet warehouse scanner. 2. Attempt to scan physical item barcode or GRN batch QR code to add line to cart.</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>Industry ERPs (SAP WM / Odoo Inventory) provide a two-step dispatch: 1) Generate Pick List from BOM/Job Order, 2) Warehouse picker marks items staged, 3) Final handover to machine operator deducts stock.</t>
+          <t>Modern ERP warehouse interfaces (Odoo Barcode app, SAP Fiori Warehouse) provide an embedded camera scanner button that instantly scans item barcodes/QR tags to add items with +1 quantity.</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>The current screen only supports a 1-step direct debit cart. There is no intermediate "Staged / Ready for Pickup" status or printable picking slip for large packaging orders.</t>
+          <t>The cart only provides a manual text search input. Storekeepers must physically type item names or alphanumeric SKUs on a keyboard, slowing down counter dispatches.</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>Mobile / Tablet</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
@@ -12459,12 +12901,12 @@
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Camera scanning built; needs a real device (Chrome on Android) — tester to verify; typed entry works everywhere.</t>
         </is>
       </c>
       <c r="M74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="N74" s="3" t="inlineStr">
@@ -12474,14 +12916,14 @@
       </c>
       <c r="O74" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed architectural gap in store issue flow (src/components/mis/store/issue-screen.tsx). The system supports only immediate 1-step direct ledger debit on cart confirm. There is no intermediate 'Staged' state, staging location tracking, or printable pick list slip for production orders.</t>
+          <t>Fail. Confirmed in ItemCart (src/components/mis/store/item-cart.tsx#L140-L165). Both issue and receive workflows rely strictly on manual keyboard search input. Neither screen provides an integrated HTML5 / WebRTC camera scanner component for mobile/tablet barcode or QR batch scanning.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>R2-78</t>
+          <t>R2-79</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -12501,32 +12943,32 @@
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Store Guy / Mobile Kiosk — Goods Issue &amp; Receive Cart (`/mis/store/issue`, `/mis/store/receive`)</t>
+          <t>Store Guy / Supervisor — Store Operations (`/mis/store/*`)</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>UI/UX Gap (ERP Standard): No integrated Barcode / 2D QR Code camera scanner in Item Cart for physical warehouse picking.</t>
+          <t>UI/UX Gap (ERP Standard): No Return-to-Store (Shop Floor Material Reversal / RMA) workflow for unused or rejected production stock.</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>1. Open `/mis/store/issue` or `/mis/store/receive` on a mobile/tablet warehouse scanner. 2. Attempt to scan physical item barcode or GRN batch QR code to add line to cart.</t>
+          <t>1. Machine operator finishes a job with 20 KG excess paper roll or unopened ink tins. 2. Attempt to return the unused material back into store inventory.</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>Modern ERP warehouse interfaces (Odoo Barcode app, SAP Fiori Warehouse) provide an embedded camera scanner button that instantly scans item barcodes/QR tags to add items with +1 quantity.</t>
+          <t>Standard manufacturing ERPs provide a formal "Return to Store / Issue Reversal" slip referencing the original Order Number/MRN, which credits inventory and reduces job actual cost.</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>The cart only provides a manual text search input. Storekeepers must physically type item names or alphanumeric SKUs on a keyboard, slowing down counter dispatches.</t>
+          <t>No Return workflow exists. Store guy must either create an ad-hoc `storeIn` (which fails to link the return back to the order or adjust job costing) or leave the balance inaccurate.</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>Mobile / Tablet</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
@@ -12536,7 +12978,7 @@
       </c>
       <c r="L75" s="3" t="inlineStr">
         <is>
-          <t>Camera scanning built; needs real-device test (Chrome/Android) — typed fallback works everywhere</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M75" s="3" t="inlineStr">
@@ -12551,14 +12993,14 @@
       </c>
       <c r="O75" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed in ItemCart (src/components/mis/store/item-cart.tsx#L140-L165). Both issue and receive workflows rely strictly on manual keyboard search input. Neither screen provides an integrated HTML5 / WebRTC camera scanner component for mobile/tablet barcode or QR batch scanning.</t>
+          <t>Fail. Confirmed architectural gap across store and order modules. There is no Return-to-Store (RTS) or issue reversal workflow in src/server/mis/store.ts or src/components/mis/store/. Unused production materials cannot be returned against an order to restore inventory balances and reduce order cost.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>R2-79</t>
+          <t>R2-80</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -12578,27 +13020,27 @@
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Store Guy / Supervisor — Store Operations (`/mis/store/*`)</t>
+          <t>Store Guy — Store Issue Screen (`/mis/store/issue`)</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>UI/UX Gap (ERP Standard): No Return-to-Store (Shop Floor Material Reversal / RMA) workflow for unused or rejected production stock.</t>
+          <t>UI/UX Gap (ERP Standard): General issues lack mandatory Cost Center / Reason Code categorization.</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>1. Machine operator finishes a job with 20 KG excess paper roll or unopened ink tins. 2. Attempt to return the unused material back into store inventory.</t>
+          <t>1. Navigate to `/mis/store/issue`. 2. Select "General issue" (no order) and "Not recorded" (no department). 3. Issue 50 units of consumable or spare parts.</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>Standard manufacturing ERPs provide a formal "Return to Store / Issue Reversal" slip referencing the original Order Number/MRN, which credits inventory and reduces job actual cost.</t>
+          <t>In SAP MM and Odoo, any stock issue not tied to a Production Work Order MUST have a mandatory Cost Center, Account Code, or Scrappage Reason (e.g. Machine Maintenance, Plant R&amp;D, Quality Scrap).</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>No Return workflow exists. Store guy must either create an ad-hoc `storeIn` (which fails to link the return back to the order or adjust job costing) or leave the balance inaccurate.</t>
+          <t>The screen allows issuing material with both Order and Department left blank, creating unallocated ledger deductions that accountants cannot attribute to any cost center.</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
@@ -12628,14 +13070,14 @@
       </c>
       <c r="O76" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed architectural gap across store and order modules. There is no Return-to-Store (RTS) or issue reversal workflow in src/server/mis/store.ts or src/components/mis/store/. Unused production materials cannot be returned against an order to restore inventory balances and reduce order cost.</t>
+          <t>Fail. Confirmed in IssueScreen (src/components/mis/store/issue-screen.tsx#L65-L85) and commitIssue (src/server/mis/store.ts). When 'General issue' is chosen, department selection defaults to 'Not recorded' and neither Cost Center nor reason code is required, allowing anonymous inventory deductions.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>R2-80</t>
+          <t>R2-81</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -12655,32 +13097,32 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Store Guy — Store Issue Screen (`/mis/store/issue`)</t>
+          <t>Admin / Owner — Supplier Invoices Screen (`/mis/supplier-invoices`)</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>UI/UX Gap (ERP Standard): General issues lack mandatory Cost Center / Reason Code categorization.</t>
+          <t>Responsiveness &amp; Layout Defect: Hardcoded `max-w-5xl` restricts desktop view instead of taking full width, while Mobile S/M/L suffers from cramped cards and filter wrapping.</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>1. Navigate to `/mis/store/issue`. 2. Select "General issue" (no order) and "Not recorded" (no department). 3. Issue 50 units of consumable or spare parts.</t>
+          <t>1. Open `/mis/supplier-invoices` on Mobile S (320px), Mobile M (375px), Mobile L (425px), and Desktop (&gt;1280px). 2. Inspect the filter chip bar, the mobile invoice cards, and the desktop 12-column match table. 3. Observe the outer layout width and responsive behavior across screen sizes.</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>In SAP MM and Odoo, any stock issue not tied to a Production Work Order MUST have a mandatory Cost Center, Account Code, or Scrappage Reason (e.g. Machine Maintenance, Plant R&amp;D, Quality Scrap).</t>
+          <t>The screen must be fully responsive across Mobile S (320px), Mobile M (375px), and Mobile L (425px) with adaptive padding and fluid card layouts. For screens greater than mobile (`&gt;= sm` / `md` / `lg` / `xl`), the layout must expand to full width (`w-full max-w-none` / `2xl:px-8`) matching the MIS desktop theme, allowing all 12 financial 3-way match columns to display legibly without squashing.</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>The screen allows issuing material with both Order and Department left blank, creating unallocated ledger deductions that accountants cannot attribute to any cost center.</t>
+          <t>The container is hardcoded to `max-w-5xl` (1024px) centered with excessive empty lateral margins on desktop, forcing the wide financial table into a cramped box. On Mobile S (320px), hardcoded `p-4` padding and fixed font sizes cause long invoice numbers and PO codes to break awkwardly.</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>All Devices (Mobile S, M, L, Tablet, Desktop)</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
@@ -12705,14 +13147,14 @@
       </c>
       <c r="O77" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed in IssueScreen (src/components/mis/store/issue-screen.tsx#L65-L85) and commitIssue (src/server/mis/store.ts). When 'General issue' is chosen, department selection defaults to 'Not recorded' and neither Cost Center nor reason code is required, allowing anonymous inventory deductions.</t>
+          <t>Fail. Confirmed in SupplierInvoicesScreen (src/components/mis/supplier-invoices/supplier-invoices-screen.tsx#L125). Outer container is locked to max-w-5xl (1024px), restricting large desktop screens from expanding to full width and causing horizontal compression of the 12-column financial matching table.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>R2-81</t>
+          <t>R2-82</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -12732,32 +13174,32 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Admin / Owner — Supplier Invoices Screen (`/mis/supplier-invoices`)</t>
+          <t>Store Guy / All Master Screens — Physical Count &amp; Master Creation Modals (`/mis/store/count`, `/mis/masters/*`)</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Responsiveness &amp; Layout Defect: Hardcoded `max-w-5xl` restricts desktop view instead of taking full width, while Mobile S/M/L suffers from cramped cards and filter wrapping.</t>
+          <t>Replace unsearchable native `&lt;select&gt;` dropdowns with shadcn `Command` Combobox for Items, Units, Machines, Operators, and Master entity selection.</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>1. Open `/mis/supplier-invoices` on Mobile S (320px), Mobile M (375px), Mobile L (425px), and Desktop (&gt;1280px). 2. Inspect the filter chip bar, the mobile invoice cards, and the desktop 12-column match table. 3. Observe the outer layout width and responsive behavior across screen sizes.</t>
+          <t>1. Navigate to Physical Count (`/mis/store/count`) and click "+ New Count" to open the sheet. 2. Inspect the "Item" selection dropdown. 3. Open any creation slide-over requiring master data (e.g., BOM stage processes, Machine board operators, Item units). 4. Attempt to quickly search and filter an item by typing.</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>The screen must be fully responsive across Mobile S (320px), Mobile M (375px), and Mobile L (425px) with adaptive padding and fluid card layouts. For screens greater than mobile (`&gt;= sm` / `md` / `lg` / `xl`), the layout must expand to full width (`w-full max-w-none` / `2xl:px-8`) matching the MIS desktop theme, allowing all 12 financial 3-way match columns to display legibly without squashing.</t>
+          <t>Master data selection (Items, Units, Machines, Operators, Processes, Suppliers) must use a searchable, keyboard-navigable combobox built on shadcn's `Command` + `Popover` component (`https://ui.shadcn.com/docs/components/base/command`), allowing instant fuzzy search across codes, SKUs, and names.</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>The container is hardcoded to `max-w-5xl` (1024px) centered with excessive empty lateral margins on desktop, forcing the wide financial table into a cramped box. On Mobile S (320px), hardcoded `p-4` padding and fixed font sizes cause long invoice numbers and PO codes to break awkwardly.</t>
+          <t>The sheet renders a native HTML `&lt;select&gt;` containing hundreds of flat `&lt;option&gt;` tags. There is no search input, filtering, or SKU highlighting. Storekeepers and operators must scroll through 200+ unsorted items manually, causing severe operational friction and wrong-item counts.</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>All Devices (Mobile S, M, L, Tablet, Desktop)</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
@@ -12767,12 +13209,12 @@
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Unit, GSM, Size, Substrate, Coating on item forms are now searchable dropdowns (inline +Add new for Admin).</t>
         </is>
       </c>
       <c r="M78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="N78" s="3" t="inlineStr">
@@ -12782,14 +13224,14 @@
       </c>
       <c r="O78" s="3" t="inlineStr">
         <is>
-          <t>Fail. Confirmed in SupplierInvoicesScreen (src/components/mis/supplier-invoices/supplier-invoices-screen.tsx#L125). Outer container is locked to max-w-5xl (1024px), restricting large desktop screens from expanding to full width and causing horizontal compression of the 12-column financial matching table.</t>
+          <t>Fail. Confirmed in StoreCountScreen (src/components/mis/store/store-count-screen.tsx#L240-L255) and master modals. Master item selection uses native unsearchable HTML &lt;select&gt; elements containing hundreds of flat &lt;option&gt; tags, lacking fuzzy search, keyboard filtering, or SKU lookup.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>R2-82</t>
+          <t>R2-83</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -12804,274 +13246,274 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Store Guy / All Master Screens — Physical Count &amp; Master Creation Modals (`/mis/store/count`, `/mis/masters/*`)</t>
+          <t>Platform Architecture / All Data Tables — PO, GRN, Invoices, Inventory, BOM, Orders, Production, QC, Payroll, Employees (`/mis/*`)</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Replace unsearchable native `&lt;select&gt;` dropdowns with shadcn `Command` Combobox for Items, Units, Machines, Operators, and Master entity selection.</t>
+          <t>Implement shadcn `Pagination` component and server-side paginated queries to eliminate unbounded data fetches and prevent DB connection pool exhaustion (`max: 1`).</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
-        <is>
-          <t>1. Navigate to Physical Count (`/mis/store/count`) and click "+ New Count" to open the sheet. 2. Inspect the "Item" selection dropdown. 3. Open any creation slide-over requiring master data (e.g., BOM stage processes, Machine board operators, Item units). 4. Attempt to quickly search and filter an item by typing.</t>
-        </is>
-      </c>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>Master data selection (Items, Units, Machines, Operators, Processes, Suppliers) must use a searchable, keyboard-navigable combobox built on shadcn's `Command` + `Popover` component (`https://ui.shadcn.com/docs/components/base/command`), allowing instant fuzzy search across codes, SKUs, and names.</t>
-        </is>
-      </c>
-      <c r="I79" s="3" t="inlineStr">
-        <is>
-          <t>The sheet renders a native HTML `&lt;select&gt;` containing hundreds of flat `&lt;option&gt;` tags. There is no search input, filtering, or SKU highlighting. Storekeepers and operators must scroll through 200+ unsorted items manually, causing severe operational friction and wrong-item counts.</t>
-        </is>
-      </c>
-      <c r="J79" s="3" t="inlineStr">
-        <is>
-          <t>Desktop / Mobile</t>
-        </is>
-      </c>
-      <c r="K79" s="3" t="inlineStr">
-        <is>
-          <t>round 2</t>
-        </is>
-      </c>
-      <c r="L79" s="3" t="inlineStr">
-        <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
-        </is>
-      </c>
-      <c r="M79" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="N79" s="3" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="O79" s="3" t="inlineStr">
-        <is>
-          <t>Fail. Confirmed in StoreCountScreen (src/components/mis/store/store-count-screen.tsx#L240-L255) and master modals. Master item selection uses native unsearchable HTML &lt;select&gt; elements containing hundreds of flat &lt;option&gt; tags, lacking fuzzy search, keyboard filtering, or SKU lookup.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="3" t="inlineStr">
-        <is>
-          <t>R2-83</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>Enhancement</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="inlineStr">
-        <is>
-          <t>Fixed - Ready to Retest</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr">
-        <is>
-          <t>Platform Architecture / All Data Tables — PO, GRN, Invoices, Inventory, BOM, Orders, Production, QC, Payroll, Employees (`/mis/*`)</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="inlineStr">
-        <is>
-          <t>Implement shadcn `Pagination` component and server-side paginated queries to eliminate unbounded data fetches and prevent DB connection pool exhaustion (`max: 1`).</t>
-        </is>
-      </c>
-      <c r="G80" s="3" t="inlineStr">
         <is>
           <t>1. Open any listing table: Purchase Orders (`/mis/po`), GRN (`/mis/grn`), Supplier Invoices (`/mis/supplier-invoices`), Orders (`/mis/orders`), Inventory (`/mis/inventory`), or Store Transactions (`/mis/store/transactions`).
 2. Observe network payload, query duration, and memory consumption as dataset grows past 500+ records.
 3. Check database connection pool metrics during concurrent queries.</t>
         </is>
       </c>
-      <c r="H80" s="3" t="inlineStr">
+      <c r="H79" s="3" t="inlineStr">
         <is>
           <t>All listing pages fetching tabular data must implement server-side pagination (with page size 25/50/100, page index, and total count) using the shadcn `Pagination` component (`https://ui.shadcn.com/docs/components/pagination`). Queries should execute `take` / `skip` in Prisma to keep queries fast, lightweight, and scalable.</t>
         </is>
       </c>
-      <c r="I80" s="3" t="inlineStr">
+      <c r="I79" s="3" t="inlineStr">
         <is>
           <t>All listing screens execute unbounded `findMany()` queries (e.g. `listStoreItems()`, `listPOs()`, `listGRNs()`, `listOrders()`) fetching entire historical datasets into memory on every page load. Because the runtime connection pool is locked to `max: 1`, unbounded queries queue behind each other, causing page latency, memory bloat, and connection timeout crashes (F-24).</t>
         </is>
       </c>
-      <c r="J80" s="3" t="inlineStr">
+      <c r="J79" s="3" t="inlineStr">
         <is>
           <t>Desktop / Mobile</t>
         </is>
       </c>
-      <c r="K80" s="3" t="inlineStr">
+      <c r="K79" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
         </is>
       </c>
-      <c r="L80" s="3" t="inlineStr">
+      <c r="L79" s="3" t="inlineStr">
         <is>
           <t>Pagination 25/page on PO, GRN, Supplier Invoices, Orders, Inventory, Employees, Audit, Store txns, Leave, Extra-pay, Daily register</t>
         </is>
       </c>
-      <c r="M80" s="3" t="inlineStr">
+      <c r="M79" s="3" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="N80" s="3" t="inlineStr">
+      <c r="N79" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="O80" s="3" t="inlineStr">
+      <c r="O79" s="3" t="inlineStr">
         <is>
           <t>Scalability bottleneck: without pagination, the single-connection database pool will freeze as live factory records accumulate.</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="3" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t>R2-84</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="C81" s="3" t="inlineStr">
+      <c r="C80" s="3" t="inlineStr">
         <is>
           <t>Fixed - Ready to Retest</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr">
+      <c r="D80" s="3" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="E81" s="3" t="inlineStr">
+      <c r="E80" s="3" t="inlineStr">
         <is>
           <t>Store &amp; Inventory — Add Item Modal (`/mis/inventory`)</t>
         </is>
       </c>
-      <c r="F81" s="3" t="inlineStr">
+      <c r="F80" s="3" t="inlineStr">
         <is>
           <t>Add Item modal on `/mis/inventory` omits Substrate and Coating fields entirely, and lacks standardized Color/Shade specification.</t>
         </is>
       </c>
-      <c r="G81" s="3" t="inlineStr">
+      <c r="G80" s="3" t="inlineStr">
         <is>
           <t>1. Navigate to `/mis/inventory` and click "+ Add Item" to open the slide-over.
 2. Inspect the fields provided (Name, Code, SKU, Category, GSM, Size, Unit, Price).
 3. Compare with Master Item Creation (`/mis/masters/items?create=1`).</t>
         </is>
       </c>
-      <c r="H81" s="3" t="inlineStr">
+      <c r="H80" s="3" t="inlineStr">
         <is>
           <t>The Add Item modal in `/mis/inventory` should match the full master schema: Substrate, Coating, GSM, Size, and Color/Shade must all be present as standardized master comboboxes so warehouse inventory records match production specs.</t>
         </is>
       </c>
-      <c r="I81" s="3" t="inlineStr">
+      <c r="I80" s="3" t="inlineStr">
         <is>
           <t>Substrate and Coating are completely absent from the `/mis/inventory` slide-over and omitted from `CreateItemInput` (`src/app/(mis)/mis/inventory/actions.ts:22-31`). Color/Shade is absent everywhere, forcing users to type redundant item names.</t>
         </is>
       </c>
-      <c r="J81" s="3" t="inlineStr">
+      <c r="J80" s="3" t="inlineStr">
         <is>
           <t>Desktop / Mobile</t>
         </is>
       </c>
-      <c r="K81" s="3" t="inlineStr">
+      <c r="K80" s="3" t="inlineStr">
         <is>
           <t>round 2</t>
         </is>
       </c>
-      <c r="L81" s="3" t="inlineStr">
+      <c r="L80" s="3" t="inlineStr">
         <is>
           <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
-      <c r="M81" s="3" t="inlineStr">
+      <c r="M80" s="3" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="N81" s="3" t="inlineStr">
+      <c r="N80" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="O81" s="3" t="inlineStr">
+      <c r="O80" s="3" t="inlineStr">
         <is>
           <t>Creates fragmented item records: items added from Inventory miss key technical specifications.</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
         <is>
           <t>R2-85</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B81" s="3" t="inlineStr">
         <is>
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr">
+      <c r="C81" s="3" t="inlineStr">
         <is>
           <t>Fixed - Ready to Retest</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr">
+      <c r="D81" s="3" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="E82" s="3" t="inlineStr">
+      <c r="E81" s="3" t="inlineStr">
         <is>
           <t>Masters &amp; Inventory — Item Creation &amp; Edit (`/mis/inventory`, `/mis/masters/items?create=1`)</t>
         </is>
       </c>
-      <c r="F82" s="3" t="inlineStr">
+      <c r="F81" s="3" t="inlineStr">
         <is>
           <t>Replace free-text inputs and native `&lt;select&gt;` with shadcn `Command` + `Popover` Combobox for Item, GSM, Size, Substrate, Coating, Color, and Unit.</t>
         </is>
       </c>
-      <c r="G82" s="3" t="inlineStr">
+      <c r="G81" s="3" t="inlineStr">
         <is>
           <t>1. Open `/mis/inventory` (Add Item) or `/mis/masters/items?create=1`.
 2. Attempt to select GSM, Size, or Unit using keyboard quick-search.
 3. Observe how Substrate and Coating are rendered (free-text inputs).</t>
         </is>
       </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>All master attributes (Item, GSM, Size, Substrate, Coating, Color, Unit) must render as searchable shadcn `Command` + `Popover` comboboxes (`https://ui.shadcn.com/docs/components/base/command`), allowing instant fuzzy search across codes and labels.</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>Substrate and Coating are rendered as unstandardized free-text `&lt;Input&gt;` fields, while GSM, Size, and Unit are native HTML `&lt;select&gt;` elements without search or filtering. Users cannot quickly type-to-filter through dozens of sizes and GSM options.</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>Desktop / Mobile</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>round 2</t>
+        </is>
+      </c>
+      <c r="L81" s="3" t="inlineStr">
+        <is>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+        </is>
+      </c>
+      <c r="M81" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="N81" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O81" s="3" t="inlineStr">
+        <is>
+          <t>Transforms item creation into a high-speed, error-free experience matching modern ERPs (SAP/Odoo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>R2-86</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Fixed - Ready to Retest</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>Admin, Owner / `/mis/employees`</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Department dropdown and field missing in Add/Edit Employee SlideOver and backend write action</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>1. Log in as Admin or Owner and navigate to `/mis/employees`. 2. Observe the "Department" column in the table. 3. Click "+ Add Employee" or "Edit" on an employee row. 4. Inspect available inputs in the slide-over form.</t>
+        </is>
+      </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>All master attributes (Item, GSM, Size, Substrate, Coating, Color, Unit) must render as searchable shadcn `Command` + `Popover` comboboxes (`https://ui.shadcn.com/docs/components/base/command`), allowing instant fuzzy search across codes and labels.</t>
+          <t>The Add/Edit Employee slide-over should render a "Department" Select dropdown populated with active departments, and createEmployee / updateEmployee in employee.ts must persist departmentId.</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>Substrate and Coating are rendered as unstandardized free-text `&lt;Input&gt;` fields, while GSM, Size, and Unit are native HTML `&lt;select&gt;` elements without search or filtering. Users cannot quickly type-to-filter through dozens of sizes and GSM options.</t>
+          <t>There is no Department input in employee-screen.tsx. In employee.ts, createEmployee and updateEmployee completely omit departmentId, leaving all employees without a department.</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>Desktop / Web</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
@@ -13081,12 +13523,12 @@
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N82" s="3" t="inlineStr">
@@ -13096,14 +13538,14 @@
       </c>
       <c r="O82" s="3" t="inlineStr">
         <is>
-          <t>Transforms item creation into a high-speed, error-free experience matching modern ERPs (SAP/Odoo).</t>
+          <t>Departmental extra-pay in payroll and machine allocation filters rely on employee.departmentId. Because it cannot be set anywhere, departmental payroll matching is broken.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>R2-86</t>
+          <t>R2-87</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -13128,27 +13570,27 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Department dropdown and field missing in Add/Edit Employee SlideOver and backend write action</t>
+          <t>One-click immediate employee deletion without confirmation dialog (useConfirm)</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as Admin or Owner and navigate to `/mis/employees`. 2. Observe the "Department" column in the table. 3. Click "+ Add Employee" or "Edit" on an employee row. 4. Inspect available inputs in the slide-over form.</t>
+          <t>1. Navigate to `/mis/employees` as Admin or Owner. 2. On any active employee row, click the "Delete" button. 3. Observe system behavior.</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>The Add/Edit Employee slide-over should render a "Department" Select dropdown populated with active departments, and createEmployee / updateEmployee in employee.ts must persist departmentId.</t>
+          <t>A destructive confirmation modal (useConfirm) should prompt: "Are you sure you want to deactivate [Employee Name]? They will no longer be able to log in or punch at the gate."</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>There is no Department input in employee-screen.tsx. In employee.ts, createEmployee and updateEmployee completely omit departmentId, leaving all employees without a department.</t>
+          <t>Clicking "Delete" immediately fires deleteEmployeeAction with zero warning or confirmation (employee-screen.tsx#L171), instantly deactivating and soft-deleting the employee.</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Web</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
@@ -13173,19 +13615,19 @@
       </c>
       <c r="O83" s="3" t="inlineStr">
         <is>
-          <t>Departmental extra-pay in payroll and machine allocation filters rely on employee.departmentId. Because it cannot be set anywhere, departmental payroll matching is broken.</t>
+          <t>In high-traffic factory floor operations, accidental clicks on mobile/touch screens cause unintended employee deactivation, locking workers out of kiosk badge scanning.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>R2-87</t>
+          <t>R2-88</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Enhancement</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -13195,32 +13637,32 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Admin, Owner / `/mis/employees`</t>
+          <t>Admin, Owner / `/mis/employees/[id]`</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>One-click immediate employee deletion without confirmation dialog (useConfirm)</t>
+          <t>Missing "Edit Employee" action button on Employee Profile Screen</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>1. Navigate to `/mis/employees` as Admin or Owner. 2. On any active employee row, click the "Delete" button. 3. Observe system behavior.</t>
+          <t>1. Navigate to `/mis/employees` and click "View" on an employee. 2. The profile screen (/mis/employees/[id]) opens. 3. Look for an "Edit Employee" button.</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>A destructive confirmation modal (useConfirm) should prompt: "Are you sure you want to deactivate [Employee Name]? They will no longer be able to log in or punch at the gate."</t>
+          <t>Administrators and Owners should have an "Edit Employee" button on the profile page to modify employee details directly.</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>Clicking "Delete" immediately fires deleteEmployeeAction with zero warning or confirmation (employee-screen.tsx#L171), instantly deactivating and soft-deleting the employee.</t>
+          <t>Only "Save photo", "Print Badge", and "Leave History" buttons exist in employee-profile-screen.tsx. Users must navigate back to the main list and locate the row to edit.</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
@@ -13235,12 +13677,12 @@
       </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N84" s="3" t="inlineStr">
@@ -13250,14 +13692,14 @@
       </c>
       <c r="O84" s="3" t="inlineStr">
         <is>
-          <t>In high-traffic factory floor operations, accidental clicks on mobile/touch screens cause unintended employee deactivation, locking workers out of kiosk badge scanning.</t>
+          <t>Disjointed navigation flow forces repetitive page bouncing between profile inspection and master editing.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>R2-88</t>
+          <t>R2-89</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -13277,32 +13719,32 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Admin, Owner / `/mis/employees/[id]`</t>
+          <t>Owner / `/mis/employees/[id]`</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>Missing "Edit Employee" action button on Employee Profile Screen</t>
+          <t>Missing link to view/print employee payslip on Employee Profile Screen</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>1. Navigate to `/mis/employees` and click "View" on an employee. 2. The profile screen (/mis/employees/[id]) opens. 3. Look for an "Edit Employee" button.</t>
+          <t>1. Log in as Owner. 2. Open an employee profile at /mis/employees/[id]. 3. Observe pay setup and attendance summary cards. 4. Look for an option to view the employee's payslip.</t>
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>Administrators and Owners should have an "Edit Employee" button on the profile page to modify employee details directly.</t>
+          <t>The Owner should have a direct quick link to view/print the employee's current payslip (/mis/print/payslip/[id]).</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Only "Save photo", "Print Badge", and "Leave History" buttons exist in employee-profile-screen.tsx. Users must navigate back to the main list and locate the row to edit.</t>
+          <t>No link to the employee's payslip exists on employee-profile-screen.tsx.</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>Desktop / Web</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
@@ -13327,19 +13769,19 @@
       </c>
       <c r="O85" s="3" t="inlineStr">
         <is>
-          <t>Disjointed navigation flow forces repetitive page bouncing between profile inspection and master editing.</t>
+          <t>The Owner has full wages.read authority; having to navigate to /mis/payroll and find the worker just to inspect their payslip is poor UX.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>R2-89</t>
+          <t>R2-90</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -13354,27 +13796,27 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Owner / `/mis/employees/[id]`</t>
+          <t>Admin, Owner, Supervisor / `/mis/employees/[id]`</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>Missing link to view/print employee payslip on Employee Profile Screen</t>
+          <t>Employee profile hardcodes current month with no month selector or historical attendance</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as Owner. 2. Open an employee profile at /mis/employees/[id]. 3. Observe pay setup and attendance summary cards. 4. Look for an option to view the employee's payslip.</t>
+          <t>1. Open /mis/employees/[id]. 2. Observe the "This Month" attendance stat card (Present, Absent, Leave, OT). 3. Attempt to view last month's stats.</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>The Owner should have a direct quick link to view/print the employee's current payslip (/mis/print/payslip/[id]).</t>
+          <t>The profile screen should provide a month selector or date controls to view past monthly attendance metrics.</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>No link to the employee's payslip exists on employee-profile-screen.tsx.</t>
+          <t>EmployeeProfilePage hardcodes new Date().getMonth() + 1 with no query parameter support (?month=) and no UI selector. Server clock new Date() also violates factory timezone D22.</t>
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr">
@@ -13389,12 +13831,12 @@
       </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N86" s="3" t="inlineStr">
@@ -13404,14 +13846,14 @@
       </c>
       <c r="O86" s="3" t="inlineStr">
         <is>
-          <t>The Owner has full wages.read authority; having to navigate to /mis/payroll and find the worker just to inspect their payslip is poor UX.</t>
+          <t>Managers cannot review historical attendance performance or trends for an employee during performance reviews or wage disputes.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>R2-90</t>
+          <t>R2-91</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -13431,27 +13873,27 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Admin, Owner, Supervisor / `/mis/employees/[id]`</t>
+          <t>Admin, Owner / `/mis/employees`</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Employee profile hardcodes current month with no month selector or historical attendance</t>
+          <t>`phone` field in `EmployeeInput` is dead code and never persisted or stored in database</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/employees/[id]. 2. Observe the "This Month" attendance stat card (Present, Absent, Leave, OT). 3. Attempt to view last month's stats.</t>
+          <t>1. Inspect src/server/mis/employee.ts. 2. Attempt to record an employee's phone number.</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>The profile screen should provide a month selector or date controls to view past monthly attendance metrics.</t>
+          <t>Employee phone numbers should be captured for emergency factory contact and SMS alerts.</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>EmployeeProfilePage hardcodes new Date().getMonth() + 1 with no query parameter support (?month=) and no UI selector. Server clock new Date() also violates factory timezone D22.</t>
+          <t>phone?: string | null is declared in EmployeeInput, but MisEmployee in prisma/schema.prisma has no phone column. Code silently drops the value.</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
@@ -13481,14 +13923,14 @@
       </c>
       <c r="O87" s="3" t="inlineStr">
         <is>
-          <t>Managers cannot review historical attendance performance or trends for an employee during performance reviews or wage disputes.</t>
+          <t>Essential HR contact information cannot be tracked anywhere in the system.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>R2-91</t>
+          <t>R2-92</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -13508,27 +13950,27 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Admin, Owner / `/mis/employees`</t>
+          <t>All Roles / `/mis/employees/[id]`</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>`phone` field in `EmployeeInput` is dead code and never persisted or stored in database</t>
+          <t>Client-side locale formatting in employee profile creates hydration mismatch and zone shift</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>1. Inspect src/server/mis/employee.ts. 2. Attempt to record an employee's phone number.</t>
+          <t>1. Set browser timezone to UTC or US Pacific. 2. Open /mis/employees/[id] for an employee registered near midnight IST. 3. Inspect the joined date.</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>Employee phone numbers should be captured for emergency factory contact and SMS alerts.</t>
+          <t>Joined date should render using formatFactoryDate(date, DEFAULT_FACTORY_TIMEZONE) in consistent factory time.</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
         <is>
-          <t>phone?: string | null is declared in EmployeeInput, but MisEmployee in prisma/schema.prisma has no phone column. Code silently drops the value.</t>
+          <t>Line 49 of employee-profile-screen.tsx uses toLocaleDateString('en-IN') in browser timezone without timeZone specifier, violating DEVELOPMENT_GUIDE §2A rule.</t>
         </is>
       </c>
       <c r="J88" s="3" t="inlineStr">
@@ -13558,14 +14000,14 @@
       </c>
       <c r="O88" s="3" t="inlineStr">
         <is>
-          <t>Essential HR contact information cannot be tracked anywhere in the system.</t>
+          <t>Causes React hydration warning in browser console and shifts joined date backwards by 1 calendar day for overseas administrators.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>R2-92</t>
+          <t>R2-93</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -13580,37 +14022,37 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>All Roles / `/mis/employees/[id]`</t>
+          <t>Attendance Operator, Admin, Owner, Supervisor / `/mis/attendance?view=daily`</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Client-side locale formatting in employee profile creates hydration mismatch and zone shift</t>
+          <t>Daily Attendance view completely lacks a date selector or day navigation controls</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>1. Set browser timezone to UTC or US Pacific. 2. Open /mis/employees/[id] for an employee registered near midnight IST. 3. Inspect the joined date.</t>
+          <t>1. Navigate to /mis/attendance?view=daily. 2. Look for date picker, calendar widget, or "Previous Day" / "Next Day" buttons. 3. Attempt to inspect yesterday's attendance.</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>Joined date should render using formatFactoryDate(date, DEFAULT_FACTORY_TIMEZONE) in consistent factory time.</t>
+          <t>The screen should provide a date input (&lt;DateInput&gt;) and Previous/Next day buttons to audit daily registers.</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Line 49 of employee-profile-screen.tsx uses toLocaleDateString('en-IN') in browser timezone without timeZone specifier, violating DEVELOPMENT_GUIDE §2A rule.</t>
+          <t>Only the Monthly tab has a month picker (attendance-screen.tsx#L160-L170). In Daily view, there are zero date navigation controls. Users are locked to factory today unless they hand-craft ?date=YYYY-MM-DD in the address bar.</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Web</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
@@ -13635,14 +14077,14 @@
       </c>
       <c r="O89" s="3" t="inlineStr">
         <is>
-          <t>Causes React hydration warning in browser console and shifts joined date backwards by 1 calendar day for overseas administrators.</t>
+          <t>Prevents attendance operators from auditing or correcting previous days' attendance without technical URL manipulation.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>R2-93</t>
+          <t>R2-94</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -13657,37 +14099,37 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Blocker</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>Attendance Operator, Admin, Owner, Supervisor / `/mis/attendance?view=daily`</t>
+          <t>Attendance Operator, Admin, Owner / `/mis/attendance`</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Daily Attendance view completely lacks a date selector or day navigation controls</t>
+          <t>Impossible to manual clock in or create attendance record for unpunched employees</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>1. Navigate to /mis/attendance?view=daily. 2. Look for date picker, calendar widget, or "Previous Day" / "Next Day" buttons. 3. Attempt to inspect yesterday's attendance.</t>
+          <t>1. Navigate to /mis/attendance?view=daily. 2. Worker arrives without a physical badge and asks the operator to clock them in manually. 3. Search for the worker in the daily register table.</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>The screen should provide a date input (&lt;DateInput&gt;) and Previous/Next day buttons to audit daily registers.</t>
+          <t>The screen should provide a "+ Manual Clock In" or "+ Add Attendance" button with an employee search dropdown to clock in any active worker.</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>Only the Monthly tab has a month picker (attendance-screen.tsx#L160-L170). In Daily view, there are zero date navigation controls. Users are locked to factory today unless they hand-craft ?date=YYYY-MM-DD in the address bar.</t>
+          <t>Table rows are derived strictly from db.misAttendance.findMany({ where: { date: d } }). Unpunched workers have no row in the database, so they DO NOT appear in the table. The "Clock In" button only exists on rows that already exist (attendance-screen.tsx:126). The operator has no way to clock them in.</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>Desktop / Web</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
@@ -13712,14 +14154,14 @@
       </c>
       <c r="O90" s="3" t="inlineStr">
         <is>
-          <t>Prevents attendance operators from auditing or correcting previous days' attendance without technical URL manipulation.</t>
+          <t>Catastrophic operational blocker: if kiosk device is offline or worker forgot badge, the operator cannot log their attendance from the web register.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>R2-94</t>
+          <t>R2-95</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -13734,7 +14176,7 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Blocker</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
@@ -13744,22 +14186,22 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>Impossible to manual clock in or create attendance record for unpunched employees</t>
+          <t>Bulk "Mark Absent" cannot select absent employees because unpunched workers have no table rows</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>1. Navigate to /mis/attendance?view=daily. 2. Worker arrives without a physical badge and asks the operator to clock them in manually. 3. Search for the worker in the daily register table.</t>
+          <t>1. At shift start, 15 workers do not show up. 2. Open /mis/attendance?view=daily. 3. Attempt to select the 15 missing workers to mark them absent in bulk.</t>
         </is>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>The screen should provide a "+ Manual Clock In" or "+ Add Attendance" button with an employee search dropdown to clock in any active worker.</t>
+          <t>The bulk selection list should include all active roster employees who do not have an attendance punch today.</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>Table rows are derived strictly from db.misAttendance.findMany({ where: { date: d } }). Unpunched workers have no row in the database, so they DO NOT appear in the table. The "Clock In" button only exists on rows that already exist (attendance-screen.tsx:126). The operator has no way to clock them in.</t>
+          <t>Checkboxes are rendered only on records (attendance-screen.tsx#L106-L116). Absent workers who never punched do not exist in records, so they cannot be selected or marked absent!</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
@@ -13789,14 +14231,14 @@
       </c>
       <c r="O91" s="3" t="inlineStr">
         <is>
-          <t>Catastrophic operational blocker: if kiosk device is offline or worker forgot badge, the operator cannot log their attendance from the web register.</t>
+          <t>Core feature failure: "Mark Absent Bulk" cannot perform its primary function of marking unrecorded absentees.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>R2-95</t>
+          <t>R2-96</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -13821,22 +14263,22 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>Bulk "Mark Absent" cannot select absent employees because unpunched workers have no table rows</t>
+          <t>Edit Attendance SlideOver lacks Clock-In and Clock-Out time pickers</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>1. At shift start, 15 workers do not show up. 2. Open /mis/attendance?view=daily. 3. Attempt to select the 15 missing workers to mark them absent in bulk.</t>
+          <t>1. On an attendance record, click "Edit". 2. SlideOver opens. 3. Inspect the input fields.</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>The bulk selection list should include all active roster employees who do not have an attendance punch today.</t>
+          <t>Operator should be able to edit and correct clockIn and clockOut times (e.g. adjust 09:35 to 09:00 if gate queue was stalled).</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>Checkboxes are rendered only on records (attendance-screen.tsx#L106-L116). Absent workers who never punched do not exist in records, so they cannot be selected or marked absent!</t>
+          <t>SlideOver only contains Status dropdown, Notes input, and Reason input (attendance-screen.tsx#L193-L208). editAttendance server function accepts clockIn and clockOut, but the UI provides no time inputs.</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
@@ -13866,14 +14308,14 @@
       </c>
       <c r="O92" s="3" t="inlineStr">
         <is>
-          <t>Core feature failure: "Mark Absent Bulk" cannot perform its primary function of marking unrecorded absentees.</t>
+          <t>Inability to adjust punch timestamps forces incorrect late penalty deductions in payroll.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>R2-96</t>
+          <t>R2-97</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -13888,32 +14330,32 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Attendance Operator, Admin, Owner / `/mis/attendance`</t>
+          <t>Admin, Owner, Attendance Operator / `/mis/attendance/shifts`</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Edit Attendance SlideOver lacks Clock-In and Clock-Out time pickers</t>
+          <t>Midnight-crossing night shifts calculate broken duration displaying "—"</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>1. On an attendance record, click "Edit". 2. SlideOver opens. 3. Inspect the input fields.</t>
+          <t>1. Navigate to /mis/attendance/shifts. 2. Create a Night Shift with Start Time 22:00 and End Time 06:00. 3. Observe the calculated duration in the list.</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>Operator should be able to edit and correct clockIn and clockOut times (e.g. adjust 09:35 to 09:00 if gate queue was stalled).</t>
+          <t>An 8-hour shift wrapping midnight (22:00 to 06:00) should display 8h 0m.</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>SlideOver only contains Status dropdown, Notes input, and Reason input (attendance-screen.tsx#L193-L208). editAttendance server function accepts clockIn and clockOut, but the UI provides no time inputs.</t>
+          <t>calcHours calculates (eh * 60 + em) - (sh * 60 + sm) = 360 - 1320 = -960. Because diff &lt;= 0, it returns '—'.</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
@@ -13943,14 +14385,14 @@
       </c>
       <c r="O93" s="3" t="inlineStr">
         <is>
-          <t>Inability to adjust punch timestamps forces incorrect late penalty deductions in payroll.</t>
+          <t>Standard manufacturing night shifts fail to render shift length in shift management cards.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>R2-97</t>
+          <t>R2-98</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -13965,7 +14407,7 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
@@ -13975,27 +14417,27 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>Midnight-crossing night shifts calculate broken duration displaying "—"</t>
+          <t>Shift Management route (`/mis/attendance/shifts`) is an unreachable orphan page</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>1. Navigate to /mis/attendance/shifts. 2. Create a Night Shift with Start Time 22:00 and End Time 06:00. 3. Observe the calculated duration in the list.</t>
+          <t>1. Log in as Admin or Owner. 2. Browse the desktop sidebar, settings menu, and attendance screens. 3. Attempt to navigate to Shift Management via UI.</t>
         </is>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>An 8-hour shift wrapping midnight (22:00 to 06:00) should display 8h 0m.</t>
+          <t>A link to "Shifts" should exist under Attendance or Settings.</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>calcHours calculates (eh * 60 + em) - (sh * 60 + sm) = 360 - 1320 = -960. Because diff &lt;= 0, it returns '—'.</t>
+          <t>Zero files in src/ link to /mis/attendance/shifts. shifts is omitted from NAV in navigation.ts#L38-L77 and omitted from attendance-screen.tsx. The screen is completely inaccessible without hand-typing the URL.</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Web</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
@@ -14020,14 +14462,14 @@
       </c>
       <c r="O94" s="3" t="inlineStr">
         <is>
-          <t>Standard manufacturing night shifts fail to render shift length in shift management cards.</t>
+          <t>Factory administrators cannot configure or adjust work shifts without developer intervention.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>R2-98</t>
+          <t>R2-99</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -14047,32 +14489,32 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Admin, Owner, Attendance Operator / `/mis/attendance/shifts`</t>
+          <t>Admin, Owner, Attendance Operator, Supervisor / Desktop Navigation</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>Shift Management route (`/mis/attendance/shifts`) is an unreachable orphan page</t>
+          <t>Leave Requests management route (`/mis/attendance/leave`) missing from desktop sidebar and attendance header</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as Admin or Owner. 2. Browse the desktop sidebar, settings menu, and attendance screens. 3. Attempt to navigate to Shift Management via UI.</t>
+          <t>1. Log in as Admin or Attendance Operator on a desktop browser. 2. Look at the desktop sidebar navigation. 3. Open /mis/attendance desktop view. 4. Look for a link to Leave Requests.</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>A link to "Shifts" should exist under Attendance or Settings.</t>
+          <t>Desktop users with attendance.read should see "Leave Requests" in the sidebar or under Attendance sub-navigation.</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>Zero files in src/ link to /mis/attendance/shifts. shifts is omitted from NAV in navigation.ts#L38-L77 and omitted from attendance-screen.tsx. The screen is completely inaccessible without hand-typing the URL.</t>
+          <t>In navigation.ts#L72, leave has phoneOnly: true, excluding it from desktop. Neither attendance-month-desktop.tsx nor attendance-screen.tsx links to /mis/attendance/leave.</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>Desktop / Web</t>
         </is>
       </c>
       <c r="K95" s="3" t="inlineStr">
@@ -14097,14 +14539,14 @@
       </c>
       <c r="O95" s="3" t="inlineStr">
         <is>
-          <t>Factory administrators cannot configure or adjust work shifts without developer intervention.</t>
+          <t>Desktop operators cannot access or process leave requests through standard navigation.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>R2-99</t>
+          <t>R2-100</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -14124,27 +14566,27 @@
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>Admin, Owner, Attendance Operator, Supervisor / Desktop Navigation</t>
+          <t>Admin, Owner, Supervisor / `/mis/employees/[id]` -&gt; `/mis/attendance/leave`</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>Leave Requests management route (`/mis/attendance/leave`) missing from desktop sidebar and attendance header</t>
+          <t>Leave History button on Employee Profile incorrectly opens create form instead of filtering leave list</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as Admin or Attendance Operator on a desktop browser. 2. Look at the desktop sidebar navigation. 3. Open /mis/attendance desktop view. 4. Look for a link to Leave Requests.</t>
+          <t>1. Open /mis/employees/[id]. 2. Click "Leave History" (/mis/attendance/leave?employeeId=...). 3. Observe the screen that opens.</t>
         </is>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>Desktop users with attendance.read should see "Leave Requests" in the sidebar or under Attendance sub-navigation.</t>
+          <t>The Leave screen should open with the table filtered to show this employee's past leave history.</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
         <is>
-          <t>In navigation.ts#L72, leave has phoneOnly: true, excluding it from desktop. Neither attendance-month-desktop.tsx nor attendance-screen.tsx links to /mis/attendance/leave.</t>
+          <t>LeaveScreen executes const [open, setOpen] = useState(!!initialEmployeeId). This automatically pops up the "Request Leave" SlideOver modal, while the table behind it remains unfiltered, showing all factory leaves.</t>
         </is>
       </c>
       <c r="J96" s="3" t="inlineStr">
@@ -14174,19 +14616,19 @@
       </c>
       <c r="O96" s="3" t="inlineStr">
         <is>
-          <t>Desktop operators cannot access or process leave requests through standard navigation.</t>
+          <t>Clicking "Leave History" confuses supervisors by popping up a new leave creation form instead of showing historical records.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>R2-100</t>
+          <t>R2-101</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Enhancement</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -14201,27 +14643,27 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Admin, Owner, Supervisor / `/mis/employees/[id]` -&gt; `/mis/attendance/leave`</t>
+          <t>Attendance Operator, Admin, Owner / `/mis/attendance/leave`</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Leave History button on Employee Profile incorrectly opens create form instead of filtering leave list</t>
+          <t>Single-day only leave requests - no date range / multi-day leave capability</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/employees/[id]. 2. Click "Leave History" (/mis/attendance/leave?employeeId=...). 3. Observe the screen that opens.</t>
+          <t>1. Open /mis/attendance/leave. 2. Click "+ Request Leave". 3. Attempt to submit a 5-day leave request for an employee.</t>
         </is>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>The Leave screen should open with the table filtered to show this employee's past leave history.</t>
+          <t>The form should support "From Date" and "To Date" range inputs to create consecutive leave days in a single submission.</t>
         </is>
       </c>
       <c r="I97" s="3" t="inlineStr">
         <is>
-          <t>LeaveScreen executes const [open, setOpen] = useState(!!initialEmployeeId). This automatically pops up the "Request Leave" SlideOver modal, while the table behind it remains unfiltered, showing all factory leaves.</t>
+          <t>Form only provides a single &lt;DateInput label="Date"&gt; (leave-screen.tsx#L149), and backend requestLeave only processes one calendar day at a time.</t>
         </is>
       </c>
       <c r="J97" s="3" t="inlineStr">
@@ -14236,12 +14678,12 @@
       </c>
       <c r="L97" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N97" s="3" t="inlineStr">
@@ -14251,14 +14693,14 @@
       </c>
       <c r="O97" s="3" t="inlineStr">
         <is>
-          <t>Clicking "Leave History" confuses supervisors by popping up a new leave creation form instead of showing historical records.</t>
+          <t>For a 10-day medical leave, the operator must manually submit 10 individual forms, and approvers must approve 10 separate rows.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>R2-101</t>
+          <t>R2-102</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -14283,22 +14725,22 @@
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>Single-day only leave requests - no date range / multi-day leave capability</t>
+          <t>Absence of standard factory leave classifications (CL, SL, EL, LWP)</t>
         </is>
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/attendance/leave. 2. Click "+ Request Leave". 3. Attempt to submit a 5-day leave request for an employee.</t>
+          <t>1. Open /mis/attendance/leave. 2. Submit a leave request. 3. Inspect leave categorization fields.</t>
         </is>
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>The form should support "From Date" and "To Date" range inputs to create consecutive leave days in a single submission.</t>
+          <t>Leave requests should allow selecting Leave Type (Casual Leave, Sick Leave, Earned Leave, Leave Without Pay).</t>
         </is>
       </c>
       <c r="I98" s="3" t="inlineStr">
         <is>
-          <t>Form only provides a single &lt;DateInput label="Date"&gt; (leave-screen.tsx#L149), and backend requestLeave only processes one calendar day at a time.</t>
+          <t>MisLeaveRequest has only reason String?. All leaves are generic text. Payroll cannot differentiate between paid statutory leave and unpaid leave.</t>
         </is>
       </c>
       <c r="J98" s="3" t="inlineStr">
@@ -14313,12 +14755,12 @@
       </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Owner can mark each leave type Paid/Unpaid in Settings &gt; Leave pay (all start Unpaid; Owner turns on Paid per type). Paid approved leave days are paid at a normal day rate in payroll; change history + audit kept.</t>
         </is>
       </c>
       <c r="M98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="N98" s="3" t="inlineStr">
@@ -14328,19 +14770,19 @@
       </c>
       <c r="O98" s="3" t="inlineStr">
         <is>
-          <t>For a 10-day medical leave, the operator must manually submit 10 individual forms, and approvers must approve 10 separate rows.</t>
+          <t>Industrial labor compliance requires tracking specific leave quotas and identifying paid vs unpaid leave for wage calculations.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>R2-102</t>
+          <t>R2-103</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -14355,32 +14797,32 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Attendance Operator, Admin, Owner / `/mis/attendance/leave`</t>
+          <t>Super Attendance Operator / `/mis` Home</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>Absence of standard factory leave classifications (CL, SL, EL, LWP)</t>
+          <t>Waive Today's Lateness card on Attendance Home is a non-functional dead UI shell</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/attendance/leave. 2. Submit a leave request. 3. Inspect leave categorization fields.</t>
+          <t>1. Log in as Super Attendance Operator. 2. On Attendance Home, toggle "Waive today's lateness" switch to ON. 3. Enter a waiver reason in the textarea. 4. Click "Apply on the register".</t>
         </is>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>Leave requests should allow selecting Leave Type (Casual Leave, Sick Leave, Earned Leave, Leave Without Pay).</t>
+          <t>The system should execute a server action waiving today's lateness for late arrivals and logging an audit event.</t>
         </is>
       </c>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>MisLeaveRequest has only reason String?. All leaves are generic text. Payroll cannot differentiate between paid statutory leave and unpaid leave.</t>
+          <t>WaiveLatenessCard holds reason in local React state. The button is a plain &lt;PrimaryButton href="/mis/attendance"&gt; link that navigates away, drops the reason, and performs zero backend mutation. /mis/attendance has no lateness waiver handler.</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Web</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K99" s="3" t="inlineStr">
@@ -14390,12 +14832,12 @@
       </c>
       <c r="L99" s="3" t="inlineStr">
         <is>
-          <t>Leave types recorded/shown; payroll does not yet differentiate paid vs unpaid leave types</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M99" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N99" s="3" t="inlineStr">
@@ -14405,14 +14847,14 @@
       </c>
       <c r="O99" s="3" t="inlineStr">
         <is>
-          <t>Industrial labor compliance requires tracking specific leave quotas and identifying paid vs unpaid leave for wage calculations.</t>
+          <t>Deceptive UI gives operators the impression lateness was waived when in reality payroll will still penalize workers for lateness.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>R2-103</t>
+          <t>R2-104</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -14427,32 +14869,32 @@
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Super Attendance Operator / `/mis` Home</t>
+          <t>Attendance Operator, Super Attendance Operator / `/mis` Home</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>Waive Today's Lateness card on Attendance Home is a non-functional dead UI shell</t>
+          <t>Reported `punchesToday` count on Attendance Home equals headcount present, not total punches</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as Super Attendance Operator. 2. On Attendance Home, toggle "Waive today's lateness" switch to ON. 3. Enter a waiver reason in the textarea. 4. Click "Apply on the register".</t>
+          <t>1. On a day with 30 present employees (who clocked in and clocked out = 60 punches), open Attendance Home. 2. Inspect the Kiosk Health Card's "punches today" metric.</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>The system should execute a server action waiving today's lateness for late arrivals and logging an audit event.</t>
+          <t>The card should report the actual count of punch events recorded today (MisAttendancePunch.count).</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
         <is>
-          <t>WaiveLatenessCard holds reason in local React state. The button is a plain &lt;PrimaryButton href="/mis/attendance"&gt; link that navigates away, drops the reason, and performs zero backend mutation. /mis/attendance has no lateness waiver handler.</t>
+          <t>Line 362 of src/app/(mis)/mis/page.tsx hardcodes const punchesToday = today.present;. It reports the headcount of present workers rather than the number of punches.</t>
         </is>
       </c>
       <c r="J100" s="3" t="inlineStr">
@@ -14482,19 +14924,19 @@
       </c>
       <c r="O100" s="3" t="inlineStr">
         <is>
-          <t>Deceptive UI gives operators the impression lateness was waived when in reality payroll will still penalize workers for lateness.</t>
+          <t>Inaccurate telemetry reporting; underreports gate tablet throughput by ~50%.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>R2-104</t>
+          <t>R2-105</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Enhancement</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -14504,37 +14946,37 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Attendance Operator, Super Attendance Operator / `/mis` Home</t>
+          <t>Attendance Operator, Admin, Owner / `/mis/kiosk`</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>Reported `punchesToday` count on Attendance Home equals headcount present, not total punches</t>
+          <t>Lack of camera/barcode/QR scanner integration on Web Kiosk Screen</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>1. On a day with 30 present employees (who clocked in and clocked out = 60 punches), open Attendance Home. 2. Inspect the Kiosk Health Card's "punches today" metric.</t>
+          <t>1. Open Web Kiosk at /mis/kiosk. 2. Attempt to scan an employee's physical badge via barcode scanner or webcam.</t>
         </is>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>The card should report the actual count of punch events recorded today (MisAttendancePunch.count).</t>
+          <t>The web kiosk should support camera barcode/QR scanning (using HTML5 video/zxing) or an autofocus HID scanner listener to auto-punch scanned badge codes.</t>
         </is>
       </c>
       <c r="I101" s="3" t="inlineStr">
         <is>
-          <t>Line 362 of src/app/(mis)/mis/page.tsx hardcodes const punchesToday = today.present;. It reports the headcount of present workers rather than the number of punches.</t>
+          <t>kiosk-screen.tsx only contains a manual text search input. The operator must manually type the worker's name or code and click through cards.</t>
         </is>
       </c>
       <c r="J101" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>Desktop / Web</t>
         </is>
       </c>
       <c r="K101" s="3" t="inlineStr">
@@ -14544,12 +14986,12 @@
       </c>
       <c r="L101" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Camera scanning built; needs a real device (Chrome on Android) — tester to verify; typed entry works everywhere.</t>
         </is>
       </c>
       <c r="M101" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="N101" s="3" t="inlineStr">
@@ -14559,19 +15001,19 @@
       </c>
       <c r="O101" s="3" t="inlineStr">
         <is>
-          <t>Inaccurate telemetry reporting; underreports gate tablet throughput by ~50%.</t>
+          <t>During peak shift changes with 100+ workers arriving simultaneously, manual keyboard search creates unmanageable gate bottlenecks.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>R2-105</t>
+          <t>R2-106</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -14581,37 +15023,37 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Blocker</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>Attendance Operator, Admin, Owner / `/mis/kiosk`</t>
+          <t>System / Attendance &amp; Payroll Integration</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Lack of camera/barcode/QR scanner integration on Web Kiosk Screen</t>
+          <t>Overtime minutes and Late minutes are never automatically derived from ingested punches</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>1. Open Web Kiosk at /mis/kiosk. 2. Attempt to scan an employee's physical badge via barcode scanner or webcam.</t>
+          <t>1. A worker assigned to shift 09:00–18:00 punches in at 09:45 (45 min late) and punches out at 20:00 (120 min OT). 2. Inspect the resulting MisAttendance record and /mis/payroll.</t>
         </is>
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>The web kiosk should support camera barcode/QR scanning (using HTML5 video/zxing) or an autofocus HID scanner listener to auto-punch scanned badge codes.</t>
+          <t>The system should calculate and record lateMinutes = 45 and otMinutes = 120 from punch timestamps against shift windows.</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
         <is>
-          <t>kiosk-screen.tsx only contains a manual text search input. The operator must manually type the worker's name or code and click through cards.</t>
+          <t>applyPunch explicitly states: // lateMinutes and otMinutes are deliberately absent (D20). The punch ingestion pipeline NEVER calculates lateMinutes or otMinutes. They remain permanently 0 unless manually updated. Consequently, payroll OT pay and late penalties always calculate as ₹0!</t>
         </is>
       </c>
       <c r="J102" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Web</t>
+          <t>Server / All</t>
         </is>
       </c>
       <c r="K102" s="3" t="inlineStr">
@@ -14621,12 +15063,12 @@
       </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
-          <t>Camera scanning built; needs real-device test (Chrome/Android) — typed fallback works everywhere</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N102" s="3" t="inlineStr">
@@ -14636,14 +15078,14 @@
       </c>
       <c r="O102" s="3" t="inlineStr">
         <is>
-          <t>During peak shift changes with 100+ workers arriving simultaneously, manual keyboard search creates unmanageable gate bottlenecks.</t>
+          <t>Critical architectural defect: real-world punches will never yield overtime wages or late penalties in payroll without automated computation.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>R2-106</t>
+          <t>R2-107</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -14658,37 +15100,37 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Blocker</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>System / Attendance &amp; Payroll Integration</t>
+          <t>Owner / `/mis/payroll` &amp; `/mis/print/payslip/[id]`</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Overtime minutes and Late minutes are never automatically derived from ingested punches</t>
+          <t>Gross Salary can calculate as negative due to uncapped late penalties and missing zero floor</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>1. A worker assigned to shift 09:00–18:00 punches in at 09:45 (45 min late) and punches out at 20:00 (120 min OT). 2. Inspect the resulting MisAttendance record and /mis/payroll.</t>
+          <t>1. In test or live setup, set an employee with 1 half-day or low basic pay. 2. Worker has multiple late arrivals resulting in late penalty exceeding basic pay. 3. Calculate monthly payroll or inspect payslip.</t>
         </is>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>The system should calculate and record lateMinutes = 45 and otMinutes = 120 from punch timestamps against shift windows.</t>
+          <t>Gross salary / Net wage should never fall below zero (Math.max(0, computedPay)).</t>
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr">
         <is>
-          <t>applyPunch explicitly states: // lateMinutes and otMinutes are deliberately absent (D20). The punch ingestion pipeline NEVER calculates lateMinutes or otMinutes. They remain permanently 0 unless manually updated. Consequently, payroll OT pay and late penalties always calculate as ₹0!</t>
+          <t>In payroll.ts:223, grossPay = basicWageOn + otPayOn + hra + allowance + bonus + extraPay - latePenaltyTotal;. Because there is no zero floor, grossPay computes as a negative number (e.g. -₹350), which renders on payslips and reports as negative income.</t>
         </is>
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
-          <t>Server / All</t>
+          <t>Desktop / Web</t>
         </is>
       </c>
       <c r="K103" s="3" t="inlineStr">
@@ -14713,14 +15155,14 @@
       </c>
       <c r="O103" s="3" t="inlineStr">
         <is>
-          <t>Critical architectural defect: real-world punches will never yield overtime wages or late penalties in payroll without automated computation.</t>
+          <t>Negative payroll violates labor regulations (Payment of Wages Act) and breaks downstream accounting exports.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>R2-107</t>
+          <t>R2-108</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -14735,32 +15177,32 @@
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>Owner / `/mis/payroll` &amp; `/mis/print/payslip/[id]`</t>
+          <t>Owner / `/mis/print/payslip/[employeeId]`</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>Gross Salary can calculate as negative due to uncapped late penalties and missing zero floor</t>
+          <t>Misleading "NET SALARY" label on payslip while displaying gross earnings without statutory deductions</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>1. In test or live setup, set an employee with 1 half-day or low basic pay. 2. Worker has multiple late arrivals resulting in late penalty exceeding basic pay. 3. Calculate monthly payroll or inspect payslip.</t>
+          <t>1. Open any employee payslip at /mis/print/payslip/[id]. 2. Look at the bottom totals row.</t>
         </is>
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>Gross salary / Net wage should never fall below zero (Math.max(0, computedPay)).</t>
+          <t>Payslip should accurately display Gross Earnings, Statutory Deductions (PF, ESI, TDS, Advance), and Net Payable Salary.</t>
         </is>
       </c>
       <c r="I104" s="3" t="inlineStr">
         <is>
-          <t>In payroll.ts:223, grossPay = basicWageOn + otPayOn + hra + allowance + bonus + extraPay - latePenaltyTotal;. Because there is no zero floor, grossPay computes as a negative number (e.g. -₹350), which renders on payslips and reports as negative income.</t>
+          <t>Line 168 of payslip/[employeeId]/page.tsx labels payroll.grossPay as "NET SALARY". In reality, no statutory deductions exist in the model. Labelling gross pay as net pay misrepresents payroll disbursements.</t>
         </is>
       </c>
       <c r="J104" s="3" t="inlineStr">
@@ -14790,19 +15232,19 @@
       </c>
       <c r="O104" s="3" t="inlineStr">
         <is>
-          <t>Negative payroll violates labor regulations (Payment of Wages Act) and breaks downstream accounting exports.</t>
+          <t>Compliance and legal vulnerability: generating official wage slips labelled "Net Salary" without statutory deduction breakdowns causes audit friction.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>R2-108</t>
+          <t>R2-109</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Enhancement</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -14817,27 +15259,27 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>Owner / `/mis/print/payslip/[employeeId]`</t>
+          <t>Owner / `/mis/payroll`</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Misleading "NET SALARY" label on payslip while displaying gross earnings without statutory deductions</t>
+          <t>Absence of bulk payslip download or batch print functionality</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>1. Open any employee payslip at /mis/print/payslip/[id]. 2. Look at the bottom totals row.</t>
+          <t>1. Open /mis/payroll at month-end. 2. Observe the employee ledger with 70+ staff. 3. Attempt to print or export payslips for all staff.</t>
         </is>
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>Payslip should accurately display Gross Earnings, Statutory Deductions (PF, ESI, TDS, Advance), and Net Payable Salary.</t>
+          <t>An Owner should have a "Print All Payslips" or "Download All Payslips (PDF/ZIP)" button.</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
         <is>
-          <t>Line 168 of payslip/[employeeId]/page.tsx labels payroll.grossPay as "NET SALARY". In reality, no statutory deductions exist in the model. Labelling gross pay as net pay misrepresents payroll disbursements.</t>
+          <t>Each row has an individual "Payslip" link (payroll-screen.tsx#L268-L270). The Owner must open 70 individual tabs and trigger browser print 70 times.</t>
         </is>
       </c>
       <c r="J105" s="3" t="inlineStr">
@@ -14852,12 +15294,12 @@
       </c>
       <c r="L105" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M105" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N105" s="3" t="inlineStr">
@@ -14867,19 +15309,19 @@
       </c>
       <c r="O105" s="3" t="inlineStr">
         <is>
-          <t>Compliance and legal vulnerability: generating official wage slips labelled "Net Salary" without statutory deduction breakdowns causes audit friction.</t>
+          <t>Unusable administrative bottleneck at monthly salary distribution for plant operations.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>R2-109</t>
+          <t>R2-110</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -14899,22 +15341,22 @@
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>Absence of bulk payslip download or batch print functionality</t>
+          <t>Month-End Payroll Export only downloads attendance counts - no wage ledger or bank transfer export</t>
         </is>
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/payroll at month-end. 2. Observe the employee ledger with 70+ staff. 3. Attempt to print or export payslips for all staff.</t>
+          <t>1. Open /mis/payroll as Owner. 2. Click "Export [Month]". 3. Open the downloaded CSV file.</t>
         </is>
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>An Owner should have a "Print All Payslips" or "Download All Payslips (PDF/ZIP)" button.</t>
+          <t>The Owner (holding wages.read) should be offered an export of the actual Financial Wage Ledger (Employee Code, Name, Basic, HRA, OT, Gross) and Bank NEFT/RTGS Transfer format.</t>
         </is>
       </c>
       <c r="I106" s="3" t="inlineStr">
         <is>
-          <t>Each row has an individual "Payslip" link (payroll-screen.tsx#L268-L270). The Owner must open 70 individual tabs and trigger browser print 70 times.</t>
+          <t>downloadCountsCsv only exports attendance numbers (Present, Absent, Leave, Half-Day, OT Hours). There is no option to export rupee amounts or bank upload files. The badge claims "XLSX (as CSV)", but it only generates count CSVs.</t>
         </is>
       </c>
       <c r="J106" s="3" t="inlineStr">
@@ -14944,14 +15386,14 @@
       </c>
       <c r="O106" s="3" t="inlineStr">
         <is>
-          <t>Unusable administrative bottleneck at monthly salary distribution for plant operations.</t>
+          <t>Plant finance teams cannot process bank payroll disbursals without wage amount exports.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>R2-110</t>
+          <t>R2-111</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -14971,32 +15413,32 @@
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>Owner / `/mis/payroll`</t>
+          <t>Supervisor, Admin, QC, Attendance Operator / `/mis/print/payslip/[employeeId]`</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>Month-End Payroll Export only downloads attendance counts - no wage ledger or bank transfer export</t>
+          <t>Logged-in employees and line managers cannot view or download their own salary slip</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/payroll as Owner. 2. Click "Export [Month]". 3. Open the downloaded CSV file.</t>
+          <t>1. Log in as a Supervisor, Admin, or Attendance Operator. 2. Locate your own employee ID. 3. Attempt to open your own payslip at /mis/print/payslip/[own-id].</t>
         </is>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>The Owner (holding wages.read) should be offered an export of the actual Financial Wage Ledger (Employee Code, Name, Basic, HRA, OT, Gross) and Bank NEFT/RTGS Transfer format.</t>
+          <t>An employee with login credentials should be permitted to view and print their OWN personal payslip.</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
         <is>
-          <t>downloadCountsCsv only exports attendance numbers (Present, Absent, Leave, Half-Day, OT Hours). There is no option to export rupee amounts or bank upload files. The badge claims "XLSX (as CSV)", but it only generates count CSVs.</t>
+          <t>PayslipPage:37 throws MisForbiddenError('wages.read') for all non-Owner roles. Non-Owner employees are completely locked out of viewing their own compensation.</t>
         </is>
       </c>
       <c r="J107" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Web</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K107" s="3" t="inlineStr">
@@ -15021,14 +15463,14 @@
       </c>
       <c r="O107" s="3" t="inlineStr">
         <is>
-          <t>Plant finance teams cannot process bank payroll disbursals without wage amount exports.</t>
+          <t>Standard HRMS self-service requirement: every employed user has the right to inspect their personal wage slip.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>R2-111</t>
+          <t>R2-112</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -15048,32 +15490,32 @@
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>Supervisor, Admin, QC, Attendance Operator / `/mis/print/payslip/[employeeId]`</t>
+          <t>Owner / `/mis/print/payslip/[employeeId]`</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>Logged-in employees and line managers cannot view or download their own salary slip</t>
+          <t>Severe performance bottleneck: individual payslip page recalculates entire factory payroll</t>
         </is>
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>1. Log in as a Supervisor, Admin, or Attendance Operator. 2. Locate your own employee ID. 3. Attempt to open your own payslip at /mis/print/payslip/[own-id].</t>
+          <t>1. Open /mis/print/payslip/[employeeId]. 2. Monitor server database queries.</t>
         </is>
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>An employee with login credentials should be permitted to view and print their OWN personal payslip.</t>
+          <t>Generating an individual worker's payslip should query only that employee's attendance and wage history.</t>
         </is>
       </c>
       <c r="I108" s="3" t="inlineStr">
         <is>
-          <t>PayslipPage:37 throws MisForbiddenError('wages.read') for all non-Owner roles. Non-Owner employees are completely locked out of viewing their own compensation.</t>
+          <t>Line 47 of payslip/[employeeId]/page.tsx executes calculateMonthlyPayroll(year, month). This recalculates all attendance and wage rules for every employee in the factory just to display one person's slip.</t>
         </is>
       </c>
       <c r="J108" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Mobile</t>
+          <t>Server / Web</t>
         </is>
       </c>
       <c r="K108" s="3" t="inlineStr">
@@ -15083,12 +15525,12 @@
       </c>
       <c r="L108" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N108" s="3" t="inlineStr">
@@ -15098,14 +15540,14 @@
       </c>
       <c r="O108" s="3" t="inlineStr">
         <is>
-          <t>Standard HRMS self-service requirement: every employed user has the right to inspect their personal wage slip.</t>
+          <t>As factory headcount scales, opening individual payslips will cause severe database CPU load and connection pool timeouts.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>R2-112</t>
+          <t>R2-113</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -15125,32 +15567,32 @@
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>Owner / `/mis/print/payslip/[employeeId]`</t>
+          <t>Owner / `/mis/settings/wages`</t>
         </is>
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Severe performance bottleneck: individual payslip page recalculates entire factory payroll</t>
+          <t>Hourly and Piece Rate wage types allowed in UI but unimplemented in payroll engine</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/print/payslip/[employeeId]. 2. Monitor server database queries.</t>
+          <t>1. Open /mis/settings/wages. 2. Click "+ Add wage type". 3. Select Unit as Hourly or Piece rate and save. 4. Assign code to an employee and run payroll.</t>
         </is>
       </c>
       <c r="H109" s="3" t="inlineStr">
         <is>
-          <t>Generating an individual worker's payslip should query only that employee's attendance and wage history.</t>
+          <t>Wage units offered in the master configuration must be fully supported by the payroll computation engine and employee pay type enum.</t>
         </is>
       </c>
       <c r="I109" s="3" t="inlineStr">
         <is>
-          <t>Line 47 of payslip/[employeeId]/page.tsx executes calculateMonthlyPayroll(year, month). This recalculates all attendance and wage rules for every employee in the factory just to display one person's slip.</t>
+          <t>UNIT_OPTIONS offers HOURLY and PIECE_RATE. But MisEmployee.payType only accepts DAILY or MONTHLY (schema.prisma#L365). In payroll.ts:135, computeEmployeeMonth has zero support for piece rate or hourly base pay, calculating erroneous figures.</t>
         </is>
       </c>
       <c r="J109" s="3" t="inlineStr">
         <is>
-          <t>Server / Web</t>
+          <t>Desktop / Web</t>
         </is>
       </c>
       <c r="K109" s="3" t="inlineStr">
@@ -15175,19 +15617,19 @@
       </c>
       <c r="O109" s="3" t="inlineStr">
         <is>
-          <t>As factory headcount scales, opening individual payslips will cause severe database CPU load and connection pool timeouts.</t>
+          <t>Creating unsupported wage codes produces broken and misleading wage calculations for piece-rate workers.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>R2-113</t>
+          <t>R2-114</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Enhancement</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -15197,7 +15639,7 @@
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="E110" s="3" t="inlineStr">
@@ -15207,22 +15649,22 @@
       </c>
       <c r="F110" s="3" t="inlineStr">
         <is>
-          <t>Hourly and Piece Rate wage types allowed in UI but unimplemented in payroll engine</t>
+          <t>Missing edit capabilities for wage type metadata and hidden historical rate revisions</t>
         </is>
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/settings/wages. 2. Click "+ Add wage type". 3. Select Unit as Hourly or Piece rate and save. 4. Assign code to an employee and run payroll.</t>
+          <t>1. Open /mis/settings/wages. 2. Observe the wage types table. 3. Try to rename a wage type or view its rate change history over past quarters.</t>
         </is>
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>Wage units offered in the master configuration must be fully supported by the payroll computation engine and employee pay type enum.</t>
+          <t>The table should offer an "Edit" button for metadata and a "History" popover showing effective date revision logs.</t>
         </is>
       </c>
       <c r="I110" s="3" t="inlineStr">
         <is>
-          <t>UNIT_OPTIONS offers HOURLY and PIECE_RATE. But MisEmployee.payType only accepts DAILY or MONTHLY (schema.prisma#L365). In payroll.ts:135, computeEmployeeMonth has zero support for piece rate or hourly base pay, calculating erroneous figures.</t>
+          <t>Table only provides "Deactivate/Reactivate" and "+ Update a rate" (wage-type-screen.tsx#L183-L188). The UI only displays the current rate row; historical revisions stored in MisWageType cannot be viewed in the UI.</t>
         </is>
       </c>
       <c r="J110" s="3" t="inlineStr">
@@ -15237,12 +15679,12 @@
       </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N110" s="3" t="inlineStr">
@@ -15252,19 +15694,19 @@
       </c>
       <c r="O110" s="3" t="inlineStr">
         <is>
-          <t>Creating unsupported wage codes produces broken and misleading wage calculations for piece-rate workers.</t>
+          <t>Factory owners cannot audit when or why wage rates were revised in previous quarters.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>R2-114</t>
+          <t>R2-115</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -15274,32 +15716,32 @@
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>Owner / `/mis/settings/wages`</t>
+          <t>Admin, Super Attendance Operator, Owner / `/mis/attendance/extra-pay`</t>
         </is>
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>Missing edit capabilities for wage type metadata and hidden historical rate revisions</t>
+          <t>Departments extra-pay scope is excluded in Propose Extra-Pay Day form</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/settings/wages. 2. Observe the wage types table. 3. Try to rename a wage type or view its rate change history over past quarters.</t>
+          <t>1. Open /mis/attendance/extra-pay. 2. Click the "Who" dropdown. 3. Observe available options.</t>
         </is>
       </c>
       <c r="H111" s="3" t="inlineStr">
         <is>
-          <t>The table should offer an "Edit" button for metadata and a "History" popover showing effective date revision logs.</t>
+          <t>The dropdown should offer "Specific department" (DEPARTMENTS), allowing bonuses for an entire team (e.g. Printing, Corrugation).</t>
         </is>
       </c>
       <c r="I111" s="3" t="inlineStr">
         <is>
-          <t>Table only provides "Deactivate/Reactivate" and "+ Update a rate" (wage-type-screen.tsx#L183-L188). The UI only displays the current rate row; historical revisions stored in MisWageType cannot be viewed in the UI.</t>
+          <t>Comment in extra-pay-propose-screen.tsx#L13-L17 notes DEPARTMENTS scope is excluded. Backend proposeExtraPayDay and payroll.ts:211 support it, but the UI omits the scope entirely.</t>
         </is>
       </c>
       <c r="J111" s="3" t="inlineStr">
@@ -15314,12 +15756,12 @@
       </c>
       <c r="L111" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
+          <t>Fixed in R2 fix batch</t>
         </is>
       </c>
       <c r="M111" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="N111" s="3" t="inlineStr">
@@ -15329,19 +15771,19 @@
       </c>
       <c r="O111" s="3" t="inlineStr">
         <is>
-          <t>Factory owners cannot audit when or why wage rates were revised in previous quarters.</t>
+          <t>Feature disconnect: backend and database support departmental extra pay, but the UI blocks users from utilizing it.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>R2-115</t>
+          <t>R2-116</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Enhancement</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -15351,7 +15793,7 @@
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="E112" s="3" t="inlineStr">
@@ -15361,27 +15803,27 @@
       </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>Departments extra-pay scope is excluded in Propose Extra-Pay Day form</t>
+          <t>Missing search filter and proposer tracking for Extra-Pay Day proposals</t>
         </is>
       </c>
       <c r="G112" s="3" t="inlineStr">
         <is>
-          <t>1. Open /mis/attendance/extra-pay. 2. Click the "Who" dropdown. 3. Observe available options.</t>
+          <t>1. Open /mis/attendance/extra-pay and select "Who" as "Specific employees". 2. Notice the employee list. 3. Submit a proposal.</t>
         </is>
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>The dropdown should offer "Specific department" (DEPARTMENTS), allowing bonuses for an entire team (e.g. Printing, Corrugation).</t>
+          <t>The employee list should include a search input and "Select All" toggle; after submission, the proposer should see a tracking table of pending/approved proposals.</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
         <is>
-          <t>Comment in extra-pay-propose-screen.tsx#L13-L17 notes DEPARTMENTS scope is excluded. Backend proposeExtraPayDay and payroll.ts:211 support it, but the UI omits the scope entirely.</t>
+          <t>The employee checkbox list has no search filter (extra-pay-propose-screen.tsx#L113-L121). After submission, the page resets to a blank form with no record or status of past proposals.</t>
         </is>
       </c>
       <c r="J112" s="3" t="inlineStr">
         <is>
-          <t>Desktop / Web</t>
+          <t>Desktop / Mobile</t>
         </is>
       </c>
       <c r="K112" s="3" t="inlineStr">
@@ -15391,12 +15833,12 @@
       </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
-          <t>Fixed in R2 fix batch</t>
+          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
         </is>
       </c>
       <c r="M112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N112" s="3" t="inlineStr">
@@ -15405,83 +15847,6 @@
         </is>
       </c>
       <c r="O112" s="3" t="inlineStr">
-        <is>
-          <t>Feature disconnect: backend and database support departmental extra pay, but the UI blocks users from utilizing it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>R2-116</t>
-        </is>
-      </c>
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t>Enhancement</t>
-        </is>
-      </c>
-      <c r="C113" s="3" t="inlineStr">
-        <is>
-          <t>Fixed - Ready to Retest</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="E113" s="3" t="inlineStr">
-        <is>
-          <t>Admin, Super Attendance Operator, Owner / `/mis/attendance/extra-pay`</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
-          <t>Missing search filter and proposer tracking for Extra-Pay Day proposals</t>
-        </is>
-      </c>
-      <c r="G113" s="3" t="inlineStr">
-        <is>
-          <t>1. Open /mis/attendance/extra-pay and select "Who" as "Specific employees". 2. Notice the employee list. 3. Submit a proposal.</t>
-        </is>
-      </c>
-      <c r="H113" s="3" t="inlineStr">
-        <is>
-          <t>The employee list should include a search input and "Select All" toggle; after submission, the proposer should see a tracking table of pending/approved proposals.</t>
-        </is>
-      </c>
-      <c r="I113" s="3" t="inlineStr">
-        <is>
-          <t>The employee checkbox list has no search filter (extra-pay-propose-screen.tsx#L113-L121). After submission, the page resets to a blank form with no record or status of past proposals.</t>
-        </is>
-      </c>
-      <c r="J113" s="3" t="inlineStr">
-        <is>
-          <t>Desktop / Mobile</t>
-        </is>
-      </c>
-      <c r="K113" s="3" t="inlineStr">
-        <is>
-          <t>round 2</t>
-        </is>
-      </c>
-      <c r="L113" s="3" t="inlineStr">
-        <is>
-          <t>Fixed in R2 batch 2 — see docs/qa/R2_DECISIONS.md</t>
-        </is>
-      </c>
-      <c r="M113" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="N113" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="O113" s="3" t="inlineStr">
         <is>
           <t>Proposers have zero visibility into whether the Owner approved or rejected their extra-pay requests.</t>
         </is>

</xml_diff>